<commit_message>
Correction to shipping AVLo values
</commit_message>
<xml_diff>
--- a/InputData/trans/AVLo/Avg Vehicle Loading.xlsx
+++ b/InputData/trans/AVLo/Avg Vehicle Loading.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\kjh_local\NEXTgroup_local\2025_local\2. EPS\업데이트 파일\eps-southkorea-3.3.1_2025update_v4.0.3\InputData\trans\AVLo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary Francis Swint\Vensim\eps-southkorea\InputData\trans\AVLo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D9CE87F-D73D-400A-A29E-6C6447025D72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D3AA79A-D381-40D7-A157-050D908BC7FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-37260" yWindow="-4620" windowWidth="28800" windowHeight="15225" firstSheet="8" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -1869,22 +1869,22 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="10">
-    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="176" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="177" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="178" formatCode="0.0"/>
-    <numFmt numFmtId="179" formatCode="###0.00_)"/>
-    <numFmt numFmtId="180" formatCode="#,##0_)"/>
-    <numFmt numFmtId="181" formatCode="#,##0_ "/>
-    <numFmt numFmtId="182" formatCode="0.00_ "/>
-    <numFmt numFmtId="183" formatCode="0.0_ "/>
-    <numFmt numFmtId="184" formatCode="0_ "/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="###0.00_)"/>
+    <numFmt numFmtId="167" formatCode="#,##0_)"/>
+    <numFmt numFmtId="168" formatCode="#,##0_ "/>
+    <numFmt numFmtId="169" formatCode="0.00_ "/>
+    <numFmt numFmtId="170" formatCode="0.0_ "/>
+    <numFmt numFmtId="171" formatCode="0_ "/>
   </numFmts>
   <fonts count="60">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1892,7 +1892,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1900,14 +1900,14 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -2129,28 +2129,28 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -2245,14 +2245,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -3038,33 +3038,33 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="177" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="177" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="179" fontId="13" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0">
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="179" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0">
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="180" fontId="15" fillId="0" borderId="5">
+    <xf numFmtId="167" fontId="15" fillId="0" borderId="5">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="16" fillId="0" borderId="5">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="13" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0">
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -3207,7 +3207,7 @@
     <xf numFmtId="49" fontId="16" fillId="0" borderId="5">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="179" fontId="15" fillId="0" borderId="0" applyNumberFormat="0">
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="0" applyNumberFormat="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="28" borderId="0">
@@ -3255,7 +3255,7 @@
     <xf numFmtId="49" fontId="33" fillId="0" borderId="5">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -3267,7 +3267,7 @@
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -3289,7 +3289,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
@@ -3304,7 +3304,7 @@
     <xf numFmtId="0" fontId="0" fillId="30" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="0" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="29" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -3319,7 +3319,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
@@ -3356,14 +3356,14 @@
     <xf numFmtId="0" fontId="48" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="48" fillId="0" borderId="19" xfId="154" applyFont="1" applyBorder="1">
+    <xf numFmtId="164" fontId="48" fillId="0" borderId="19" xfId="154" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="48" fillId="33" borderId="19" xfId="154" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="164" fontId="48" fillId="33" borderId="19" xfId="154" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="182" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="183" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="41" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3376,7 +3376,7 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
@@ -3413,30 +3413,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="43" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="43" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="184" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="184" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="184" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="184" fontId="0" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="0" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -3529,8 +3529,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="30" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3539,7 +3539,7 @@
     <xf numFmtId="0" fontId="58" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="184" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3603,6 +3603,7 @@
     <cellStyle name="Calculation 2" xfId="29" xr:uid="{00000000-0005-0000-0000-00001B000000}"/>
     <cellStyle name="Check Cell 2" xfId="30" xr:uid="{00000000-0005-0000-0000-00001C000000}"/>
     <cellStyle name="Column heading" xfId="31" xr:uid="{00000000-0005-0000-0000-00001D000000}"/>
+    <cellStyle name="Comma [0]" xfId="154" builtinId="6"/>
     <cellStyle name="Comma 2" xfId="32" xr:uid="{00000000-0005-0000-0000-00001E000000}"/>
     <cellStyle name="Comma 2 2" xfId="33" xr:uid="{00000000-0005-0000-0000-00001F000000}"/>
     <cellStyle name="Comma 3" xfId="34" xr:uid="{00000000-0005-0000-0000-000020000000}"/>
@@ -3641,10 +3642,12 @@
     <cellStyle name="Hed Top" xfId="67" xr:uid="{00000000-0005-0000-0000-000041000000}"/>
     <cellStyle name="Hed Top - SECTION" xfId="68" xr:uid="{00000000-0005-0000-0000-000042000000}"/>
     <cellStyle name="Hed Top_3-new4" xfId="69" xr:uid="{00000000-0005-0000-0000-000043000000}"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Hyperlink 2" xfId="70" xr:uid="{00000000-0005-0000-0000-000045000000}"/>
     <cellStyle name="Input 2" xfId="71" xr:uid="{00000000-0005-0000-0000-000046000000}"/>
     <cellStyle name="Linked Cell 2" xfId="72" xr:uid="{00000000-0005-0000-0000-000047000000}"/>
     <cellStyle name="Neutral 2" xfId="73" xr:uid="{00000000-0005-0000-0000-000048000000}"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 10" xfId="74" xr:uid="{00000000-0005-0000-0000-00004A000000}"/>
     <cellStyle name="Normal 11" xfId="75" xr:uid="{00000000-0005-0000-0000-00004B000000}"/>
     <cellStyle name="Normal 2" xfId="76" xr:uid="{00000000-0005-0000-0000-00004C000000}"/>
@@ -3725,9 +3728,6 @@
     <cellStyle name="Wrap Bold" xfId="151" xr:uid="{00000000-0005-0000-0000-000097000000}"/>
     <cellStyle name="Wrap Title" xfId="152" xr:uid="{00000000-0005-0000-0000-000098000000}"/>
     <cellStyle name="Wrap_NTS99-~11" xfId="153" xr:uid="{00000000-0005-0000-0000-000099000000}"/>
-    <cellStyle name="쉼표 [0]" xfId="154" builtinId="6"/>
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
-    <cellStyle name="하이퍼링크" xfId="1" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -4390,10 +4390,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F42"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="11.5" customWidth="1"/>
-    <col min="2" max="2" width="85.125" customWidth="1"/>
+    <col min="1" max="1" width="11.453125" customWidth="1"/>
+    <col min="2" max="2" width="85.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -4640,7 +4640,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4E8B5F8-CAC2-4F37-8597-58946AEA5DB1}">
   <dimension ref="A1:U25"/>
-  <sheetFormatPr defaultColWidth="19" defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultColWidth="19" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
   </cols>
@@ -5607,8 +5607,8 @@
         <v>44536.615934699075</v>
       </c>
     </row>
-    <row r="19" spans="1:21" ht="17.25" thickBot="1"/>
-    <row r="20" spans="1:21" ht="17.25" thickBot="1">
+    <row r="19" spans="1:21" ht="15" thickBot="1"/>
+    <row r="20" spans="1:21" ht="15" thickBot="1">
       <c r="A20" s="106"/>
       <c r="B20" s="107" t="s">
         <v>426</v>
@@ -5617,7 +5617,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="21" spans="1:21" ht="17.25" thickTop="1">
+    <row r="21" spans="1:21" ht="15" thickTop="1">
       <c r="A21" s="109" t="s">
         <v>423</v>
       </c>
@@ -5640,7 +5640,7 @@
         <v>0.48580480150021893</v>
       </c>
     </row>
-    <row r="23" spans="1:21" ht="17.25" thickBot="1">
+    <row r="23" spans="1:21" ht="15" thickBot="1">
       <c r="A23" s="82" t="s">
         <v>425</v>
       </c>
@@ -5671,13 +5671,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9438158E-C803-4774-ADE5-31C8503BC4B7}">
   <dimension ref="A1:Q31"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="3" width="14.875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.875" customWidth="1"/>
+    <col min="2" max="3" width="14.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="17.25" thickBot="1">
+    <row r="1" spans="1:9" ht="15" thickBot="1">
       <c r="A1" s="27" t="s">
         <v>342</v>
       </c>
@@ -5701,7 +5701,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="17.25" thickBot="1">
+    <row r="3" spans="1:9" ht="15" thickBot="1">
       <c r="A3" s="103"/>
       <c r="B3" s="85"/>
       <c r="C3" s="130" t="s">
@@ -5717,7 +5717,7 @@
       <c r="G3" s="85"/>
       <c r="H3" s="86"/>
     </row>
-    <row r="4" spans="1:9" ht="17.25" thickTop="1">
+    <row r="4" spans="1:9" ht="15" thickTop="1">
       <c r="A4" s="100" t="s">
         <v>381</v>
       </c>
@@ -5780,7 +5780,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="17.25" thickBot="1">
+    <row r="7" spans="1:9" ht="15" thickBot="1">
       <c r="A7" s="103"/>
       <c r="B7" s="104"/>
       <c r="C7" s="104"/>
@@ -5793,7 +5793,7 @@
       <c r="H7" s="105"/>
       <c r="I7" s="44"/>
     </row>
-    <row r="8" spans="1:9" ht="17.25" thickTop="1">
+    <row r="8" spans="1:9" ht="15" thickTop="1">
       <c r="A8" s="100" t="s">
         <v>380</v>
       </c>
@@ -5817,7 +5817,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="17.25" thickBot="1">
+    <row r="9" spans="1:9" ht="15" thickBot="1">
       <c r="A9" s="82"/>
       <c r="B9" s="102" t="s">
         <v>383</v>
@@ -5843,7 +5843,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="17.25">
+    <row r="11" spans="1:9" ht="17.5">
       <c r="B11" s="76" t="s">
         <v>378</v>
       </c>
@@ -5919,7 +5919,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="28" spans="1:17" ht="17.25" thickBot="1">
+    <row r="28" spans="1:17" ht="15" thickBot="1">
       <c r="A28" s="7" t="s">
         <v>282</v>
       </c>
@@ -5927,7 +5927,7 @@
       <c r="C28" s="8"/>
       <c r="D28" s="8"/>
     </row>
-    <row r="29" spans="1:17" ht="17.25" thickBot="1">
+    <row r="29" spans="1:17" ht="15" thickBot="1">
       <c r="A29" s="93"/>
       <c r="B29" s="94" t="s">
         <v>56</v>
@@ -5942,7 +5942,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="30" spans="1:17" ht="17.25" thickTop="1">
+    <row r="30" spans="1:17" ht="15" thickTop="1">
       <c r="A30" s="90" t="s">
         <v>59</v>
       </c>
@@ -5961,7 +5961,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="31" spans="1:17" ht="17.25" thickBot="1">
+    <row r="31" spans="1:17" ht="15" thickBot="1">
       <c r="A31" s="87" t="s">
         <v>60</v>
       </c>
@@ -5993,7 +5993,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8AABE4-9A7A-4FF9-8C38-25844DE09CA8}">
   <dimension ref="A1:AK15"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:37">
       <c r="A1" t="s">
@@ -7568,13 +7568,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AK7"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="13.125" customWidth="1"/>
-    <col min="2" max="2" width="8.75" customWidth="1"/>
+    <col min="1" max="1" width="13.08984375" customWidth="1"/>
+    <col min="2" max="2" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" ht="49.5">
+    <row r="1" spans="1:37" ht="43.5">
       <c r="A1" s="6" t="s">
         <v>9</v>
       </c>
@@ -7798,7 +7798,8 @@
         <v>6</v>
       </c>
       <c r="B6" s="4">
-        <v>1</v>
+        <f>'ships-psgr'!G3</f>
+        <v>337.61417769892506</v>
       </c>
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
@@ -7891,12 +7892,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AJ7"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="11.875" customWidth="1"/>
+    <col min="1" max="1" width="11.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" s="1" customFormat="1" ht="49.5">
+    <row r="1" spans="1:36" s="1" customFormat="1" ht="43.5">
       <c r="A1" s="6" t="s">
         <v>10</v>
       </c>
@@ -8106,13 +8107,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AK7"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="13.125" customWidth="1"/>
-    <col min="2" max="2" width="8.75" customWidth="1"/>
+    <col min="1" max="1" width="13.08984375" customWidth="1"/>
+    <col min="2" max="2" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" ht="49.5">
+    <row r="1" spans="1:37" ht="43.5">
       <c r="A1" s="6" t="s">
         <v>9</v>
       </c>
@@ -8826,112 +8827,148 @@
         <v>6</v>
       </c>
       <c r="B6" s="4">
-        <v>1</v>
+        <f>'ships-psgr'!G3</f>
+        <v>337.61417769892506</v>
       </c>
       <c r="C6" s="4">
-        <v>1</v>
+        <f>B6</f>
+        <v>337.61417769892506</v>
       </c>
       <c r="D6" s="4">
-        <v>1</v>
+        <f t="shared" ref="D6:AK6" si="2">C6</f>
+        <v>337.61417769892506</v>
       </c>
       <c r="E6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="F6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="G6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="H6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="I6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="J6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="K6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="L6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="M6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="N6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="O6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="P6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="Q6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="R6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="S6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="T6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="U6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="V6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="W6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="X6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="Y6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="Z6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="AA6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="AB6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="AC6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="AD6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="AE6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="AF6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="AG6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="AH6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="AI6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="AJ6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
       <c r="AK6" s="4">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>337.61417769892506</v>
       </c>
     </row>
     <row r="7" spans="1:37">
@@ -9094,12 +9131,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AJ7"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="11.875" customWidth="1"/>
+    <col min="1" max="1" width="11.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" s="1" customFormat="1" ht="49.5">
+    <row r="1" spans="1:36" s="1" customFormat="1" ht="43.5">
       <c r="A1" s="6" t="s">
         <v>10</v>
       </c>
@@ -10088,10 +10125,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6E22F11-BE45-4915-A8C3-90BE8CB5DD1C}">
   <dimension ref="A39:I61"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="3" max="3" width="12.875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="39" spans="2:9">
@@ -10278,20 +10315,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46AB8DE8-67C3-4E44-9B0E-EF6D34DD1C9C}">
   <dimension ref="A1:W142"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="4" style="29" customWidth="1"/>
-    <col min="2" max="2" width="3.5" style="29" customWidth="1"/>
-    <col min="3" max="4" width="1.5" style="29" customWidth="1"/>
-    <col min="5" max="5" width="23.25" style="29" customWidth="1"/>
-    <col min="6" max="9" width="11.5" style="29" hidden="1" customWidth="1"/>
-    <col min="10" max="12" width="10.125" style="29" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="10.5" style="29" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="11.5" style="29" hidden="1" customWidth="1"/>
-    <col min="15" max="19" width="10.125" style="29" hidden="1" customWidth="1"/>
-    <col min="20" max="21" width="11.5" style="29" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="10.125" style="29" hidden="1" customWidth="1"/>
-    <col min="23" max="23" width="12.5" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.453125" style="29" customWidth="1"/>
+    <col min="3" max="4" width="1.453125" style="29" customWidth="1"/>
+    <col min="5" max="5" width="23.26953125" style="29" customWidth="1"/>
+    <col min="6" max="9" width="11.453125" style="29" hidden="1" customWidth="1"/>
+    <col min="10" max="12" width="10.08984375" style="29" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="10.453125" style="29" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="11.453125" style="29" hidden="1" customWidth="1"/>
+    <col min="15" max="19" width="10.08984375" style="29" hidden="1" customWidth="1"/>
+    <col min="20" max="21" width="11.453125" style="29" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="10.08984375" style="29" hidden="1" customWidth="1"/>
+    <col min="23" max="23" width="12.453125" style="29" bestFit="1" customWidth="1"/>
     <col min="24" max="16384" width="9" style="29"/>
   </cols>
   <sheetData>
@@ -19135,13 +19172,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAD3B914-B72F-432B-8D51-3CBE259118E1}">
   <dimension ref="J2:P18"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="11" width="9" style="8"/>
-    <col min="12" max="12" width="10.875" style="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.90625" style="8" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="9" style="8"/>
-    <col min="14" max="14" width="16.25" style="8" customWidth="1"/>
-    <col min="15" max="15" width="18.5" style="8" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.26953125" style="8" customWidth="1"/>
+    <col min="15" max="15" width="18.453125" style="8" bestFit="1" customWidth="1"/>
     <col min="16" max="16384" width="9" style="8"/>
   </cols>
   <sheetData>
@@ -19283,23 +19320,23 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{152A55CB-ED11-48EF-AA99-B206FDDEB829}">
   <dimension ref="A1:P51"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="9" style="8"/>
-    <col min="2" max="2" width="13.125" style="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.875" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.875" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.75" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.125" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.08984375" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.90625" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.90625" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.7265625" style="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.08984375" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.453125" style="8" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9" style="8"/>
     <col min="9" max="9" width="11" style="8" customWidth="1"/>
-    <col min="10" max="10" width="12.25" style="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.875" style="8" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.125" style="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.875" style="8" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17.75" style="8" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.75" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.26953125" style="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.90625" style="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.08984375" style="8" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.90625" style="8" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.7265625" style="8" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.7265625" style="8" bestFit="1" customWidth="1"/>
     <col min="16" max="16384" width="9" style="8"/>
   </cols>
   <sheetData>
@@ -20802,16 +20839,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DBB0CBB-759C-4C56-A4C4-D4E65F9775FA}">
   <dimension ref="B2:I175"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="10.75" customWidth="1"/>
-    <col min="5" max="5" width="15.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7265625" customWidth="1"/>
+    <col min="5" max="5" width="15.90625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19" customWidth="1"/>
-    <col min="7" max="7" width="20.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.5" customWidth="1"/>
+    <col min="7" max="7" width="20.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" ht="17.25" thickBot="1">
+    <row r="2" spans="2:9" ht="15" thickBot="1">
       <c r="B2" s="53" t="s">
         <v>271</v>
       </c>
@@ -20925,7 +20962,7 @@
         <v>254.87619047619049</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="17.25" thickBot="1">
+    <row r="8" spans="2:9" ht="15" thickBot="1">
       <c r="B8" s="27" t="s">
         <v>265</v>
       </c>
@@ -20962,7 +20999,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="13" spans="2:9" ht="17.25" thickBot="1">
+    <row r="13" spans="2:9" ht="15" thickBot="1">
       <c r="B13" s="53" t="s">
         <v>271</v>
       </c>
@@ -21112,7 +21149,7 @@
         <v>254.87619047619049</v>
       </c>
     </row>
-    <row r="19" spans="2:9" ht="17.25" thickBot="1">
+    <row r="19" spans="2:9" ht="15" thickBot="1">
       <c r="B19" t="s">
         <v>263</v>
       </c>
@@ -22869,11 +22906,11 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACC9CD64-51B3-4C21-ABDF-5DD1D16C3DC4}">
   <dimension ref="A1:H29"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="16.5" customWidth="1"/>
-    <col min="3" max="4" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.5" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
+    <col min="3" max="4" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.453125" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
   </cols>
   <sheetData>
@@ -22882,7 +22919,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="17.25" thickBot="1">
+    <row r="2" spans="1:7" ht="15" thickBot="1">
       <c r="A2" s="116" t="s">
         <v>446</v>
       </c>
@@ -23286,7 +23323,7 @@
         <v>45.8</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="17.25" thickBot="1">
+    <row r="21" spans="1:8" ht="15" thickBot="1">
       <c r="A21" s="104" t="s">
         <v>468</v>
       </c>
@@ -23304,7 +23341,7 @@
         <v>25406.090909090908</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="17.25" thickTop="1">
+    <row r="22" spans="1:8" ht="15" thickTop="1">
       <c r="A22" s="115" t="s">
         <v>54</v>
       </c>
@@ -23338,7 +23375,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="17.25" thickBot="1">
+    <row r="25" spans="1:8" ht="15" thickBot="1">
       <c r="A25" s="123" t="s">
         <v>471</v>
       </c>
@@ -23475,27 +23512,27 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{834C8993-7EE0-4137-9B77-501005A3F9D6}">
   <dimension ref="A2:N49"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="11.75" style="8" customWidth="1"/>
+    <col min="1" max="1" width="11.7265625" style="8" customWidth="1"/>
     <col min="2" max="2" width="9" style="8"/>
-    <col min="3" max="4" width="11.5" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.875" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="11.453125" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.90625" style="8" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="9" style="8"/>
-    <col min="8" max="8" width="8.875" style="8" customWidth="1"/>
-    <col min="9" max="9" width="12.5" style="8" customWidth="1"/>
-    <col min="10" max="10" width="3.75" style="8" customWidth="1"/>
-    <col min="11" max="11" width="4.5" style="8" customWidth="1"/>
-    <col min="12" max="12" width="20.25" style="8" customWidth="1"/>
+    <col min="8" max="8" width="8.90625" style="8" customWidth="1"/>
+    <col min="9" max="9" width="12.453125" style="8" customWidth="1"/>
+    <col min="10" max="10" width="3.7265625" style="8" customWidth="1"/>
+    <col min="11" max="11" width="4.453125" style="8" customWidth="1"/>
+    <col min="12" max="12" width="20.26953125" style="8" customWidth="1"/>
     <col min="13" max="13" width="17" style="8" customWidth="1"/>
     <col min="14" max="14" width="18" style="8" customWidth="1"/>
     <col min="15" max="16" width="9" style="8"/>
-    <col min="17" max="17" width="11.125" style="8" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.25" style="8" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.08984375" style="8" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.26953125" style="8" bestFit="1" customWidth="1"/>
     <col min="19" max="16384" width="9" style="8"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" ht="17.25" thickBot="1">
+    <row r="2" spans="2:12" ht="15" thickBot="1">
       <c r="D2" s="56" t="s">
         <v>300</v>
       </c>
@@ -23766,7 +23803,7 @@
         <v>43669</v>
       </c>
     </row>
-    <row r="16" spans="2:12" ht="17.25" thickBot="1">
+    <row r="16" spans="2:12" ht="15" thickBot="1">
       <c r="B16" s="62">
         <v>2018</v>
       </c>
@@ -24760,456 +24797,456 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08F5C122-988D-446F-A1DB-C3D7ACE874B7}">
   <dimension ref="A1:R23"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="21.125" customWidth="1"/>
-    <col min="2" max="2" width="12.5" customWidth="1"/>
-    <col min="3" max="7" width="12.75" customWidth="1"/>
-    <col min="8" max="8" width="12.875" customWidth="1"/>
-    <col min="9" max="10" width="12.75" customWidth="1"/>
-    <col min="11" max="14" width="12.875" customWidth="1"/>
-    <col min="15" max="18" width="12.75" customWidth="1"/>
-    <col min="257" max="257" width="21.125" customWidth="1"/>
-    <col min="258" max="258" width="12.5" customWidth="1"/>
-    <col min="259" max="263" width="12.75" customWidth="1"/>
-    <col min="264" max="264" width="12.875" customWidth="1"/>
-    <col min="265" max="266" width="12.75" customWidth="1"/>
-    <col min="267" max="270" width="12.875" customWidth="1"/>
-    <col min="271" max="274" width="12.75" customWidth="1"/>
-    <col min="513" max="513" width="21.125" customWidth="1"/>
-    <col min="514" max="514" width="12.5" customWidth="1"/>
-    <col min="515" max="519" width="12.75" customWidth="1"/>
-    <col min="520" max="520" width="12.875" customWidth="1"/>
-    <col min="521" max="522" width="12.75" customWidth="1"/>
-    <col min="523" max="526" width="12.875" customWidth="1"/>
-    <col min="527" max="530" width="12.75" customWidth="1"/>
-    <col min="769" max="769" width="21.125" customWidth="1"/>
-    <col min="770" max="770" width="12.5" customWidth="1"/>
-    <col min="771" max="775" width="12.75" customWidth="1"/>
-    <col min="776" max="776" width="12.875" customWidth="1"/>
-    <col min="777" max="778" width="12.75" customWidth="1"/>
-    <col min="779" max="782" width="12.875" customWidth="1"/>
-    <col min="783" max="786" width="12.75" customWidth="1"/>
-    <col min="1025" max="1025" width="21.125" customWidth="1"/>
-    <col min="1026" max="1026" width="12.5" customWidth="1"/>
-    <col min="1027" max="1031" width="12.75" customWidth="1"/>
-    <col min="1032" max="1032" width="12.875" customWidth="1"/>
-    <col min="1033" max="1034" width="12.75" customWidth="1"/>
-    <col min="1035" max="1038" width="12.875" customWidth="1"/>
-    <col min="1039" max="1042" width="12.75" customWidth="1"/>
-    <col min="1281" max="1281" width="21.125" customWidth="1"/>
-    <col min="1282" max="1282" width="12.5" customWidth="1"/>
-    <col min="1283" max="1287" width="12.75" customWidth="1"/>
-    <col min="1288" max="1288" width="12.875" customWidth="1"/>
-    <col min="1289" max="1290" width="12.75" customWidth="1"/>
-    <col min="1291" max="1294" width="12.875" customWidth="1"/>
-    <col min="1295" max="1298" width="12.75" customWidth="1"/>
-    <col min="1537" max="1537" width="21.125" customWidth="1"/>
-    <col min="1538" max="1538" width="12.5" customWidth="1"/>
-    <col min="1539" max="1543" width="12.75" customWidth="1"/>
-    <col min="1544" max="1544" width="12.875" customWidth="1"/>
-    <col min="1545" max="1546" width="12.75" customWidth="1"/>
-    <col min="1547" max="1550" width="12.875" customWidth="1"/>
-    <col min="1551" max="1554" width="12.75" customWidth="1"/>
-    <col min="1793" max="1793" width="21.125" customWidth="1"/>
-    <col min="1794" max="1794" width="12.5" customWidth="1"/>
-    <col min="1795" max="1799" width="12.75" customWidth="1"/>
-    <col min="1800" max="1800" width="12.875" customWidth="1"/>
-    <col min="1801" max="1802" width="12.75" customWidth="1"/>
-    <col min="1803" max="1806" width="12.875" customWidth="1"/>
-    <col min="1807" max="1810" width="12.75" customWidth="1"/>
-    <col min="2049" max="2049" width="21.125" customWidth="1"/>
-    <col min="2050" max="2050" width="12.5" customWidth="1"/>
-    <col min="2051" max="2055" width="12.75" customWidth="1"/>
-    <col min="2056" max="2056" width="12.875" customWidth="1"/>
-    <col min="2057" max="2058" width="12.75" customWidth="1"/>
-    <col min="2059" max="2062" width="12.875" customWidth="1"/>
-    <col min="2063" max="2066" width="12.75" customWidth="1"/>
-    <col min="2305" max="2305" width="21.125" customWidth="1"/>
-    <col min="2306" max="2306" width="12.5" customWidth="1"/>
-    <col min="2307" max="2311" width="12.75" customWidth="1"/>
-    <col min="2312" max="2312" width="12.875" customWidth="1"/>
-    <col min="2313" max="2314" width="12.75" customWidth="1"/>
-    <col min="2315" max="2318" width="12.875" customWidth="1"/>
-    <col min="2319" max="2322" width="12.75" customWidth="1"/>
-    <col min="2561" max="2561" width="21.125" customWidth="1"/>
-    <col min="2562" max="2562" width="12.5" customWidth="1"/>
-    <col min="2563" max="2567" width="12.75" customWidth="1"/>
-    <col min="2568" max="2568" width="12.875" customWidth="1"/>
-    <col min="2569" max="2570" width="12.75" customWidth="1"/>
-    <col min="2571" max="2574" width="12.875" customWidth="1"/>
-    <col min="2575" max="2578" width="12.75" customWidth="1"/>
-    <col min="2817" max="2817" width="21.125" customWidth="1"/>
-    <col min="2818" max="2818" width="12.5" customWidth="1"/>
-    <col min="2819" max="2823" width="12.75" customWidth="1"/>
-    <col min="2824" max="2824" width="12.875" customWidth="1"/>
-    <col min="2825" max="2826" width="12.75" customWidth="1"/>
-    <col min="2827" max="2830" width="12.875" customWidth="1"/>
-    <col min="2831" max="2834" width="12.75" customWidth="1"/>
-    <col min="3073" max="3073" width="21.125" customWidth="1"/>
-    <col min="3074" max="3074" width="12.5" customWidth="1"/>
-    <col min="3075" max="3079" width="12.75" customWidth="1"/>
-    <col min="3080" max="3080" width="12.875" customWidth="1"/>
-    <col min="3081" max="3082" width="12.75" customWidth="1"/>
-    <col min="3083" max="3086" width="12.875" customWidth="1"/>
-    <col min="3087" max="3090" width="12.75" customWidth="1"/>
-    <col min="3329" max="3329" width="21.125" customWidth="1"/>
-    <col min="3330" max="3330" width="12.5" customWidth="1"/>
-    <col min="3331" max="3335" width="12.75" customWidth="1"/>
-    <col min="3336" max="3336" width="12.875" customWidth="1"/>
-    <col min="3337" max="3338" width="12.75" customWidth="1"/>
-    <col min="3339" max="3342" width="12.875" customWidth="1"/>
-    <col min="3343" max="3346" width="12.75" customWidth="1"/>
-    <col min="3585" max="3585" width="21.125" customWidth="1"/>
-    <col min="3586" max="3586" width="12.5" customWidth="1"/>
-    <col min="3587" max="3591" width="12.75" customWidth="1"/>
-    <col min="3592" max="3592" width="12.875" customWidth="1"/>
-    <col min="3593" max="3594" width="12.75" customWidth="1"/>
-    <col min="3595" max="3598" width="12.875" customWidth="1"/>
-    <col min="3599" max="3602" width="12.75" customWidth="1"/>
-    <col min="3841" max="3841" width="21.125" customWidth="1"/>
-    <col min="3842" max="3842" width="12.5" customWidth="1"/>
-    <col min="3843" max="3847" width="12.75" customWidth="1"/>
-    <col min="3848" max="3848" width="12.875" customWidth="1"/>
-    <col min="3849" max="3850" width="12.75" customWidth="1"/>
-    <col min="3851" max="3854" width="12.875" customWidth="1"/>
-    <col min="3855" max="3858" width="12.75" customWidth="1"/>
-    <col min="4097" max="4097" width="21.125" customWidth="1"/>
-    <col min="4098" max="4098" width="12.5" customWidth="1"/>
-    <col min="4099" max="4103" width="12.75" customWidth="1"/>
-    <col min="4104" max="4104" width="12.875" customWidth="1"/>
-    <col min="4105" max="4106" width="12.75" customWidth="1"/>
-    <col min="4107" max="4110" width="12.875" customWidth="1"/>
-    <col min="4111" max="4114" width="12.75" customWidth="1"/>
-    <col min="4353" max="4353" width="21.125" customWidth="1"/>
-    <col min="4354" max="4354" width="12.5" customWidth="1"/>
-    <col min="4355" max="4359" width="12.75" customWidth="1"/>
-    <col min="4360" max="4360" width="12.875" customWidth="1"/>
-    <col min="4361" max="4362" width="12.75" customWidth="1"/>
-    <col min="4363" max="4366" width="12.875" customWidth="1"/>
-    <col min="4367" max="4370" width="12.75" customWidth="1"/>
-    <col min="4609" max="4609" width="21.125" customWidth="1"/>
-    <col min="4610" max="4610" width="12.5" customWidth="1"/>
-    <col min="4611" max="4615" width="12.75" customWidth="1"/>
-    <col min="4616" max="4616" width="12.875" customWidth="1"/>
-    <col min="4617" max="4618" width="12.75" customWidth="1"/>
-    <col min="4619" max="4622" width="12.875" customWidth="1"/>
-    <col min="4623" max="4626" width="12.75" customWidth="1"/>
-    <col min="4865" max="4865" width="21.125" customWidth="1"/>
-    <col min="4866" max="4866" width="12.5" customWidth="1"/>
-    <col min="4867" max="4871" width="12.75" customWidth="1"/>
-    <col min="4872" max="4872" width="12.875" customWidth="1"/>
-    <col min="4873" max="4874" width="12.75" customWidth="1"/>
-    <col min="4875" max="4878" width="12.875" customWidth="1"/>
-    <col min="4879" max="4882" width="12.75" customWidth="1"/>
-    <col min="5121" max="5121" width="21.125" customWidth="1"/>
-    <col min="5122" max="5122" width="12.5" customWidth="1"/>
-    <col min="5123" max="5127" width="12.75" customWidth="1"/>
-    <col min="5128" max="5128" width="12.875" customWidth="1"/>
-    <col min="5129" max="5130" width="12.75" customWidth="1"/>
-    <col min="5131" max="5134" width="12.875" customWidth="1"/>
-    <col min="5135" max="5138" width="12.75" customWidth="1"/>
-    <col min="5377" max="5377" width="21.125" customWidth="1"/>
-    <col min="5378" max="5378" width="12.5" customWidth="1"/>
-    <col min="5379" max="5383" width="12.75" customWidth="1"/>
-    <col min="5384" max="5384" width="12.875" customWidth="1"/>
-    <col min="5385" max="5386" width="12.75" customWidth="1"/>
-    <col min="5387" max="5390" width="12.875" customWidth="1"/>
-    <col min="5391" max="5394" width="12.75" customWidth="1"/>
-    <col min="5633" max="5633" width="21.125" customWidth="1"/>
-    <col min="5634" max="5634" width="12.5" customWidth="1"/>
-    <col min="5635" max="5639" width="12.75" customWidth="1"/>
-    <col min="5640" max="5640" width="12.875" customWidth="1"/>
-    <col min="5641" max="5642" width="12.75" customWidth="1"/>
-    <col min="5643" max="5646" width="12.875" customWidth="1"/>
-    <col min="5647" max="5650" width="12.75" customWidth="1"/>
-    <col min="5889" max="5889" width="21.125" customWidth="1"/>
-    <col min="5890" max="5890" width="12.5" customWidth="1"/>
-    <col min="5891" max="5895" width="12.75" customWidth="1"/>
-    <col min="5896" max="5896" width="12.875" customWidth="1"/>
-    <col min="5897" max="5898" width="12.75" customWidth="1"/>
-    <col min="5899" max="5902" width="12.875" customWidth="1"/>
-    <col min="5903" max="5906" width="12.75" customWidth="1"/>
-    <col min="6145" max="6145" width="21.125" customWidth="1"/>
-    <col min="6146" max="6146" width="12.5" customWidth="1"/>
-    <col min="6147" max="6151" width="12.75" customWidth="1"/>
-    <col min="6152" max="6152" width="12.875" customWidth="1"/>
-    <col min="6153" max="6154" width="12.75" customWidth="1"/>
-    <col min="6155" max="6158" width="12.875" customWidth="1"/>
-    <col min="6159" max="6162" width="12.75" customWidth="1"/>
-    <col min="6401" max="6401" width="21.125" customWidth="1"/>
-    <col min="6402" max="6402" width="12.5" customWidth="1"/>
-    <col min="6403" max="6407" width="12.75" customWidth="1"/>
-    <col min="6408" max="6408" width="12.875" customWidth="1"/>
-    <col min="6409" max="6410" width="12.75" customWidth="1"/>
-    <col min="6411" max="6414" width="12.875" customWidth="1"/>
-    <col min="6415" max="6418" width="12.75" customWidth="1"/>
-    <col min="6657" max="6657" width="21.125" customWidth="1"/>
-    <col min="6658" max="6658" width="12.5" customWidth="1"/>
-    <col min="6659" max="6663" width="12.75" customWidth="1"/>
-    <col min="6664" max="6664" width="12.875" customWidth="1"/>
-    <col min="6665" max="6666" width="12.75" customWidth="1"/>
-    <col min="6667" max="6670" width="12.875" customWidth="1"/>
-    <col min="6671" max="6674" width="12.75" customWidth="1"/>
-    <col min="6913" max="6913" width="21.125" customWidth="1"/>
-    <col min="6914" max="6914" width="12.5" customWidth="1"/>
-    <col min="6915" max="6919" width="12.75" customWidth="1"/>
-    <col min="6920" max="6920" width="12.875" customWidth="1"/>
-    <col min="6921" max="6922" width="12.75" customWidth="1"/>
-    <col min="6923" max="6926" width="12.875" customWidth="1"/>
-    <col min="6927" max="6930" width="12.75" customWidth="1"/>
-    <col min="7169" max="7169" width="21.125" customWidth="1"/>
-    <col min="7170" max="7170" width="12.5" customWidth="1"/>
-    <col min="7171" max="7175" width="12.75" customWidth="1"/>
-    <col min="7176" max="7176" width="12.875" customWidth="1"/>
-    <col min="7177" max="7178" width="12.75" customWidth="1"/>
-    <col min="7179" max="7182" width="12.875" customWidth="1"/>
-    <col min="7183" max="7186" width="12.75" customWidth="1"/>
-    <col min="7425" max="7425" width="21.125" customWidth="1"/>
-    <col min="7426" max="7426" width="12.5" customWidth="1"/>
-    <col min="7427" max="7431" width="12.75" customWidth="1"/>
-    <col min="7432" max="7432" width="12.875" customWidth="1"/>
-    <col min="7433" max="7434" width="12.75" customWidth="1"/>
-    <col min="7435" max="7438" width="12.875" customWidth="1"/>
-    <col min="7439" max="7442" width="12.75" customWidth="1"/>
-    <col min="7681" max="7681" width="21.125" customWidth="1"/>
-    <col min="7682" max="7682" width="12.5" customWidth="1"/>
-    <col min="7683" max="7687" width="12.75" customWidth="1"/>
-    <col min="7688" max="7688" width="12.875" customWidth="1"/>
-    <col min="7689" max="7690" width="12.75" customWidth="1"/>
-    <col min="7691" max="7694" width="12.875" customWidth="1"/>
-    <col min="7695" max="7698" width="12.75" customWidth="1"/>
-    <col min="7937" max="7937" width="21.125" customWidth="1"/>
-    <col min="7938" max="7938" width="12.5" customWidth="1"/>
-    <col min="7939" max="7943" width="12.75" customWidth="1"/>
-    <col min="7944" max="7944" width="12.875" customWidth="1"/>
-    <col min="7945" max="7946" width="12.75" customWidth="1"/>
-    <col min="7947" max="7950" width="12.875" customWidth="1"/>
-    <col min="7951" max="7954" width="12.75" customWidth="1"/>
-    <col min="8193" max="8193" width="21.125" customWidth="1"/>
-    <col min="8194" max="8194" width="12.5" customWidth="1"/>
-    <col min="8195" max="8199" width="12.75" customWidth="1"/>
-    <col min="8200" max="8200" width="12.875" customWidth="1"/>
-    <col min="8201" max="8202" width="12.75" customWidth="1"/>
-    <col min="8203" max="8206" width="12.875" customWidth="1"/>
-    <col min="8207" max="8210" width="12.75" customWidth="1"/>
-    <col min="8449" max="8449" width="21.125" customWidth="1"/>
-    <col min="8450" max="8450" width="12.5" customWidth="1"/>
-    <col min="8451" max="8455" width="12.75" customWidth="1"/>
-    <col min="8456" max="8456" width="12.875" customWidth="1"/>
-    <col min="8457" max="8458" width="12.75" customWidth="1"/>
-    <col min="8459" max="8462" width="12.875" customWidth="1"/>
-    <col min="8463" max="8466" width="12.75" customWidth="1"/>
-    <col min="8705" max="8705" width="21.125" customWidth="1"/>
-    <col min="8706" max="8706" width="12.5" customWidth="1"/>
-    <col min="8707" max="8711" width="12.75" customWidth="1"/>
-    <col min="8712" max="8712" width="12.875" customWidth="1"/>
-    <col min="8713" max="8714" width="12.75" customWidth="1"/>
-    <col min="8715" max="8718" width="12.875" customWidth="1"/>
-    <col min="8719" max="8722" width="12.75" customWidth="1"/>
-    <col min="8961" max="8961" width="21.125" customWidth="1"/>
-    <col min="8962" max="8962" width="12.5" customWidth="1"/>
-    <col min="8963" max="8967" width="12.75" customWidth="1"/>
-    <col min="8968" max="8968" width="12.875" customWidth="1"/>
-    <col min="8969" max="8970" width="12.75" customWidth="1"/>
-    <col min="8971" max="8974" width="12.875" customWidth="1"/>
-    <col min="8975" max="8978" width="12.75" customWidth="1"/>
-    <col min="9217" max="9217" width="21.125" customWidth="1"/>
-    <col min="9218" max="9218" width="12.5" customWidth="1"/>
-    <col min="9219" max="9223" width="12.75" customWidth="1"/>
-    <col min="9224" max="9224" width="12.875" customWidth="1"/>
-    <col min="9225" max="9226" width="12.75" customWidth="1"/>
-    <col min="9227" max="9230" width="12.875" customWidth="1"/>
-    <col min="9231" max="9234" width="12.75" customWidth="1"/>
-    <col min="9473" max="9473" width="21.125" customWidth="1"/>
-    <col min="9474" max="9474" width="12.5" customWidth="1"/>
-    <col min="9475" max="9479" width="12.75" customWidth="1"/>
-    <col min="9480" max="9480" width="12.875" customWidth="1"/>
-    <col min="9481" max="9482" width="12.75" customWidth="1"/>
-    <col min="9483" max="9486" width="12.875" customWidth="1"/>
-    <col min="9487" max="9490" width="12.75" customWidth="1"/>
-    <col min="9729" max="9729" width="21.125" customWidth="1"/>
-    <col min="9730" max="9730" width="12.5" customWidth="1"/>
-    <col min="9731" max="9735" width="12.75" customWidth="1"/>
-    <col min="9736" max="9736" width="12.875" customWidth="1"/>
-    <col min="9737" max="9738" width="12.75" customWidth="1"/>
-    <col min="9739" max="9742" width="12.875" customWidth="1"/>
-    <col min="9743" max="9746" width="12.75" customWidth="1"/>
-    <col min="9985" max="9985" width="21.125" customWidth="1"/>
-    <col min="9986" max="9986" width="12.5" customWidth="1"/>
-    <col min="9987" max="9991" width="12.75" customWidth="1"/>
-    <col min="9992" max="9992" width="12.875" customWidth="1"/>
-    <col min="9993" max="9994" width="12.75" customWidth="1"/>
-    <col min="9995" max="9998" width="12.875" customWidth="1"/>
-    <col min="9999" max="10002" width="12.75" customWidth="1"/>
-    <col min="10241" max="10241" width="21.125" customWidth="1"/>
-    <col min="10242" max="10242" width="12.5" customWidth="1"/>
-    <col min="10243" max="10247" width="12.75" customWidth="1"/>
-    <col min="10248" max="10248" width="12.875" customWidth="1"/>
-    <col min="10249" max="10250" width="12.75" customWidth="1"/>
-    <col min="10251" max="10254" width="12.875" customWidth="1"/>
-    <col min="10255" max="10258" width="12.75" customWidth="1"/>
-    <col min="10497" max="10497" width="21.125" customWidth="1"/>
-    <col min="10498" max="10498" width="12.5" customWidth="1"/>
-    <col min="10499" max="10503" width="12.75" customWidth="1"/>
-    <col min="10504" max="10504" width="12.875" customWidth="1"/>
-    <col min="10505" max="10506" width="12.75" customWidth="1"/>
-    <col min="10507" max="10510" width="12.875" customWidth="1"/>
-    <col min="10511" max="10514" width="12.75" customWidth="1"/>
-    <col min="10753" max="10753" width="21.125" customWidth="1"/>
-    <col min="10754" max="10754" width="12.5" customWidth="1"/>
-    <col min="10755" max="10759" width="12.75" customWidth="1"/>
-    <col min="10760" max="10760" width="12.875" customWidth="1"/>
-    <col min="10761" max="10762" width="12.75" customWidth="1"/>
-    <col min="10763" max="10766" width="12.875" customWidth="1"/>
-    <col min="10767" max="10770" width="12.75" customWidth="1"/>
-    <col min="11009" max="11009" width="21.125" customWidth="1"/>
-    <col min="11010" max="11010" width="12.5" customWidth="1"/>
-    <col min="11011" max="11015" width="12.75" customWidth="1"/>
-    <col min="11016" max="11016" width="12.875" customWidth="1"/>
-    <col min="11017" max="11018" width="12.75" customWidth="1"/>
-    <col min="11019" max="11022" width="12.875" customWidth="1"/>
-    <col min="11023" max="11026" width="12.75" customWidth="1"/>
-    <col min="11265" max="11265" width="21.125" customWidth="1"/>
-    <col min="11266" max="11266" width="12.5" customWidth="1"/>
-    <col min="11267" max="11271" width="12.75" customWidth="1"/>
-    <col min="11272" max="11272" width="12.875" customWidth="1"/>
-    <col min="11273" max="11274" width="12.75" customWidth="1"/>
-    <col min="11275" max="11278" width="12.875" customWidth="1"/>
-    <col min="11279" max="11282" width="12.75" customWidth="1"/>
-    <col min="11521" max="11521" width="21.125" customWidth="1"/>
-    <col min="11522" max="11522" width="12.5" customWidth="1"/>
-    <col min="11523" max="11527" width="12.75" customWidth="1"/>
-    <col min="11528" max="11528" width="12.875" customWidth="1"/>
-    <col min="11529" max="11530" width="12.75" customWidth="1"/>
-    <col min="11531" max="11534" width="12.875" customWidth="1"/>
-    <col min="11535" max="11538" width="12.75" customWidth="1"/>
-    <col min="11777" max="11777" width="21.125" customWidth="1"/>
-    <col min="11778" max="11778" width="12.5" customWidth="1"/>
-    <col min="11779" max="11783" width="12.75" customWidth="1"/>
-    <col min="11784" max="11784" width="12.875" customWidth="1"/>
-    <col min="11785" max="11786" width="12.75" customWidth="1"/>
-    <col min="11787" max="11790" width="12.875" customWidth="1"/>
-    <col min="11791" max="11794" width="12.75" customWidth="1"/>
-    <col min="12033" max="12033" width="21.125" customWidth="1"/>
-    <col min="12034" max="12034" width="12.5" customWidth="1"/>
-    <col min="12035" max="12039" width="12.75" customWidth="1"/>
-    <col min="12040" max="12040" width="12.875" customWidth="1"/>
-    <col min="12041" max="12042" width="12.75" customWidth="1"/>
-    <col min="12043" max="12046" width="12.875" customWidth="1"/>
-    <col min="12047" max="12050" width="12.75" customWidth="1"/>
-    <col min="12289" max="12289" width="21.125" customWidth="1"/>
-    <col min="12290" max="12290" width="12.5" customWidth="1"/>
-    <col min="12291" max="12295" width="12.75" customWidth="1"/>
-    <col min="12296" max="12296" width="12.875" customWidth="1"/>
-    <col min="12297" max="12298" width="12.75" customWidth="1"/>
-    <col min="12299" max="12302" width="12.875" customWidth="1"/>
-    <col min="12303" max="12306" width="12.75" customWidth="1"/>
-    <col min="12545" max="12545" width="21.125" customWidth="1"/>
-    <col min="12546" max="12546" width="12.5" customWidth="1"/>
-    <col min="12547" max="12551" width="12.75" customWidth="1"/>
-    <col min="12552" max="12552" width="12.875" customWidth="1"/>
-    <col min="12553" max="12554" width="12.75" customWidth="1"/>
-    <col min="12555" max="12558" width="12.875" customWidth="1"/>
-    <col min="12559" max="12562" width="12.75" customWidth="1"/>
-    <col min="12801" max="12801" width="21.125" customWidth="1"/>
-    <col min="12802" max="12802" width="12.5" customWidth="1"/>
-    <col min="12803" max="12807" width="12.75" customWidth="1"/>
-    <col min="12808" max="12808" width="12.875" customWidth="1"/>
-    <col min="12809" max="12810" width="12.75" customWidth="1"/>
-    <col min="12811" max="12814" width="12.875" customWidth="1"/>
-    <col min="12815" max="12818" width="12.75" customWidth="1"/>
-    <col min="13057" max="13057" width="21.125" customWidth="1"/>
-    <col min="13058" max="13058" width="12.5" customWidth="1"/>
-    <col min="13059" max="13063" width="12.75" customWidth="1"/>
-    <col min="13064" max="13064" width="12.875" customWidth="1"/>
-    <col min="13065" max="13066" width="12.75" customWidth="1"/>
-    <col min="13067" max="13070" width="12.875" customWidth="1"/>
-    <col min="13071" max="13074" width="12.75" customWidth="1"/>
-    <col min="13313" max="13313" width="21.125" customWidth="1"/>
-    <col min="13314" max="13314" width="12.5" customWidth="1"/>
-    <col min="13315" max="13319" width="12.75" customWidth="1"/>
-    <col min="13320" max="13320" width="12.875" customWidth="1"/>
-    <col min="13321" max="13322" width="12.75" customWidth="1"/>
-    <col min="13323" max="13326" width="12.875" customWidth="1"/>
-    <col min="13327" max="13330" width="12.75" customWidth="1"/>
-    <col min="13569" max="13569" width="21.125" customWidth="1"/>
-    <col min="13570" max="13570" width="12.5" customWidth="1"/>
-    <col min="13571" max="13575" width="12.75" customWidth="1"/>
-    <col min="13576" max="13576" width="12.875" customWidth="1"/>
-    <col min="13577" max="13578" width="12.75" customWidth="1"/>
-    <col min="13579" max="13582" width="12.875" customWidth="1"/>
-    <col min="13583" max="13586" width="12.75" customWidth="1"/>
-    <col min="13825" max="13825" width="21.125" customWidth="1"/>
-    <col min="13826" max="13826" width="12.5" customWidth="1"/>
-    <col min="13827" max="13831" width="12.75" customWidth="1"/>
-    <col min="13832" max="13832" width="12.875" customWidth="1"/>
-    <col min="13833" max="13834" width="12.75" customWidth="1"/>
-    <col min="13835" max="13838" width="12.875" customWidth="1"/>
-    <col min="13839" max="13842" width="12.75" customWidth="1"/>
-    <col min="14081" max="14081" width="21.125" customWidth="1"/>
-    <col min="14082" max="14082" width="12.5" customWidth="1"/>
-    <col min="14083" max="14087" width="12.75" customWidth="1"/>
-    <col min="14088" max="14088" width="12.875" customWidth="1"/>
-    <col min="14089" max="14090" width="12.75" customWidth="1"/>
-    <col min="14091" max="14094" width="12.875" customWidth="1"/>
-    <col min="14095" max="14098" width="12.75" customWidth="1"/>
-    <col min="14337" max="14337" width="21.125" customWidth="1"/>
-    <col min="14338" max="14338" width="12.5" customWidth="1"/>
-    <col min="14339" max="14343" width="12.75" customWidth="1"/>
-    <col min="14344" max="14344" width="12.875" customWidth="1"/>
-    <col min="14345" max="14346" width="12.75" customWidth="1"/>
-    <col min="14347" max="14350" width="12.875" customWidth="1"/>
-    <col min="14351" max="14354" width="12.75" customWidth="1"/>
-    <col min="14593" max="14593" width="21.125" customWidth="1"/>
-    <col min="14594" max="14594" width="12.5" customWidth="1"/>
-    <col min="14595" max="14599" width="12.75" customWidth="1"/>
-    <col min="14600" max="14600" width="12.875" customWidth="1"/>
-    <col min="14601" max="14602" width="12.75" customWidth="1"/>
-    <col min="14603" max="14606" width="12.875" customWidth="1"/>
-    <col min="14607" max="14610" width="12.75" customWidth="1"/>
-    <col min="14849" max="14849" width="21.125" customWidth="1"/>
-    <col min="14850" max="14850" width="12.5" customWidth="1"/>
-    <col min="14851" max="14855" width="12.75" customWidth="1"/>
-    <col min="14856" max="14856" width="12.875" customWidth="1"/>
-    <col min="14857" max="14858" width="12.75" customWidth="1"/>
-    <col min="14859" max="14862" width="12.875" customWidth="1"/>
-    <col min="14863" max="14866" width="12.75" customWidth="1"/>
-    <col min="15105" max="15105" width="21.125" customWidth="1"/>
-    <col min="15106" max="15106" width="12.5" customWidth="1"/>
-    <col min="15107" max="15111" width="12.75" customWidth="1"/>
-    <col min="15112" max="15112" width="12.875" customWidth="1"/>
-    <col min="15113" max="15114" width="12.75" customWidth="1"/>
-    <col min="15115" max="15118" width="12.875" customWidth="1"/>
-    <col min="15119" max="15122" width="12.75" customWidth="1"/>
-    <col min="15361" max="15361" width="21.125" customWidth="1"/>
-    <col min="15362" max="15362" width="12.5" customWidth="1"/>
-    <col min="15363" max="15367" width="12.75" customWidth="1"/>
-    <col min="15368" max="15368" width="12.875" customWidth="1"/>
-    <col min="15369" max="15370" width="12.75" customWidth="1"/>
-    <col min="15371" max="15374" width="12.875" customWidth="1"/>
-    <col min="15375" max="15378" width="12.75" customWidth="1"/>
-    <col min="15617" max="15617" width="21.125" customWidth="1"/>
-    <col min="15618" max="15618" width="12.5" customWidth="1"/>
-    <col min="15619" max="15623" width="12.75" customWidth="1"/>
-    <col min="15624" max="15624" width="12.875" customWidth="1"/>
-    <col min="15625" max="15626" width="12.75" customWidth="1"/>
-    <col min="15627" max="15630" width="12.875" customWidth="1"/>
-    <col min="15631" max="15634" width="12.75" customWidth="1"/>
-    <col min="15873" max="15873" width="21.125" customWidth="1"/>
-    <col min="15874" max="15874" width="12.5" customWidth="1"/>
-    <col min="15875" max="15879" width="12.75" customWidth="1"/>
-    <col min="15880" max="15880" width="12.875" customWidth="1"/>
-    <col min="15881" max="15882" width="12.75" customWidth="1"/>
-    <col min="15883" max="15886" width="12.875" customWidth="1"/>
-    <col min="15887" max="15890" width="12.75" customWidth="1"/>
-    <col min="16129" max="16129" width="21.125" customWidth="1"/>
-    <col min="16130" max="16130" width="12.5" customWidth="1"/>
-    <col min="16131" max="16135" width="12.75" customWidth="1"/>
-    <col min="16136" max="16136" width="12.875" customWidth="1"/>
-    <col min="16137" max="16138" width="12.75" customWidth="1"/>
-    <col min="16139" max="16142" width="12.875" customWidth="1"/>
-    <col min="16143" max="16146" width="12.75" customWidth="1"/>
+    <col min="1" max="1" width="21.08984375" customWidth="1"/>
+    <col min="2" max="2" width="12.453125" customWidth="1"/>
+    <col min="3" max="7" width="12.7265625" customWidth="1"/>
+    <col min="8" max="8" width="12.90625" customWidth="1"/>
+    <col min="9" max="10" width="12.7265625" customWidth="1"/>
+    <col min="11" max="14" width="12.90625" customWidth="1"/>
+    <col min="15" max="18" width="12.7265625" customWidth="1"/>
+    <col min="257" max="257" width="21.08984375" customWidth="1"/>
+    <col min="258" max="258" width="12.453125" customWidth="1"/>
+    <col min="259" max="263" width="12.7265625" customWidth="1"/>
+    <col min="264" max="264" width="12.90625" customWidth="1"/>
+    <col min="265" max="266" width="12.7265625" customWidth="1"/>
+    <col min="267" max="270" width="12.90625" customWidth="1"/>
+    <col min="271" max="274" width="12.7265625" customWidth="1"/>
+    <col min="513" max="513" width="21.08984375" customWidth="1"/>
+    <col min="514" max="514" width="12.453125" customWidth="1"/>
+    <col min="515" max="519" width="12.7265625" customWidth="1"/>
+    <col min="520" max="520" width="12.90625" customWidth="1"/>
+    <col min="521" max="522" width="12.7265625" customWidth="1"/>
+    <col min="523" max="526" width="12.90625" customWidth="1"/>
+    <col min="527" max="530" width="12.7265625" customWidth="1"/>
+    <col min="769" max="769" width="21.08984375" customWidth="1"/>
+    <col min="770" max="770" width="12.453125" customWidth="1"/>
+    <col min="771" max="775" width="12.7265625" customWidth="1"/>
+    <col min="776" max="776" width="12.90625" customWidth="1"/>
+    <col min="777" max="778" width="12.7265625" customWidth="1"/>
+    <col min="779" max="782" width="12.90625" customWidth="1"/>
+    <col min="783" max="786" width="12.7265625" customWidth="1"/>
+    <col min="1025" max="1025" width="21.08984375" customWidth="1"/>
+    <col min="1026" max="1026" width="12.453125" customWidth="1"/>
+    <col min="1027" max="1031" width="12.7265625" customWidth="1"/>
+    <col min="1032" max="1032" width="12.90625" customWidth="1"/>
+    <col min="1033" max="1034" width="12.7265625" customWidth="1"/>
+    <col min="1035" max="1038" width="12.90625" customWidth="1"/>
+    <col min="1039" max="1042" width="12.7265625" customWidth="1"/>
+    <col min="1281" max="1281" width="21.08984375" customWidth="1"/>
+    <col min="1282" max="1282" width="12.453125" customWidth="1"/>
+    <col min="1283" max="1287" width="12.7265625" customWidth="1"/>
+    <col min="1288" max="1288" width="12.90625" customWidth="1"/>
+    <col min="1289" max="1290" width="12.7265625" customWidth="1"/>
+    <col min="1291" max="1294" width="12.90625" customWidth="1"/>
+    <col min="1295" max="1298" width="12.7265625" customWidth="1"/>
+    <col min="1537" max="1537" width="21.08984375" customWidth="1"/>
+    <col min="1538" max="1538" width="12.453125" customWidth="1"/>
+    <col min="1539" max="1543" width="12.7265625" customWidth="1"/>
+    <col min="1544" max="1544" width="12.90625" customWidth="1"/>
+    <col min="1545" max="1546" width="12.7265625" customWidth="1"/>
+    <col min="1547" max="1550" width="12.90625" customWidth="1"/>
+    <col min="1551" max="1554" width="12.7265625" customWidth="1"/>
+    <col min="1793" max="1793" width="21.08984375" customWidth="1"/>
+    <col min="1794" max="1794" width="12.453125" customWidth="1"/>
+    <col min="1795" max="1799" width="12.7265625" customWidth="1"/>
+    <col min="1800" max="1800" width="12.90625" customWidth="1"/>
+    <col min="1801" max="1802" width="12.7265625" customWidth="1"/>
+    <col min="1803" max="1806" width="12.90625" customWidth="1"/>
+    <col min="1807" max="1810" width="12.7265625" customWidth="1"/>
+    <col min="2049" max="2049" width="21.08984375" customWidth="1"/>
+    <col min="2050" max="2050" width="12.453125" customWidth="1"/>
+    <col min="2051" max="2055" width="12.7265625" customWidth="1"/>
+    <col min="2056" max="2056" width="12.90625" customWidth="1"/>
+    <col min="2057" max="2058" width="12.7265625" customWidth="1"/>
+    <col min="2059" max="2062" width="12.90625" customWidth="1"/>
+    <col min="2063" max="2066" width="12.7265625" customWidth="1"/>
+    <col min="2305" max="2305" width="21.08984375" customWidth="1"/>
+    <col min="2306" max="2306" width="12.453125" customWidth="1"/>
+    <col min="2307" max="2311" width="12.7265625" customWidth="1"/>
+    <col min="2312" max="2312" width="12.90625" customWidth="1"/>
+    <col min="2313" max="2314" width="12.7265625" customWidth="1"/>
+    <col min="2315" max="2318" width="12.90625" customWidth="1"/>
+    <col min="2319" max="2322" width="12.7265625" customWidth="1"/>
+    <col min="2561" max="2561" width="21.08984375" customWidth="1"/>
+    <col min="2562" max="2562" width="12.453125" customWidth="1"/>
+    <col min="2563" max="2567" width="12.7265625" customWidth="1"/>
+    <col min="2568" max="2568" width="12.90625" customWidth="1"/>
+    <col min="2569" max="2570" width="12.7265625" customWidth="1"/>
+    <col min="2571" max="2574" width="12.90625" customWidth="1"/>
+    <col min="2575" max="2578" width="12.7265625" customWidth="1"/>
+    <col min="2817" max="2817" width="21.08984375" customWidth="1"/>
+    <col min="2818" max="2818" width="12.453125" customWidth="1"/>
+    <col min="2819" max="2823" width="12.7265625" customWidth="1"/>
+    <col min="2824" max="2824" width="12.90625" customWidth="1"/>
+    <col min="2825" max="2826" width="12.7265625" customWidth="1"/>
+    <col min="2827" max="2830" width="12.90625" customWidth="1"/>
+    <col min="2831" max="2834" width="12.7265625" customWidth="1"/>
+    <col min="3073" max="3073" width="21.08984375" customWidth="1"/>
+    <col min="3074" max="3074" width="12.453125" customWidth="1"/>
+    <col min="3075" max="3079" width="12.7265625" customWidth="1"/>
+    <col min="3080" max="3080" width="12.90625" customWidth="1"/>
+    <col min="3081" max="3082" width="12.7265625" customWidth="1"/>
+    <col min="3083" max="3086" width="12.90625" customWidth="1"/>
+    <col min="3087" max="3090" width="12.7265625" customWidth="1"/>
+    <col min="3329" max="3329" width="21.08984375" customWidth="1"/>
+    <col min="3330" max="3330" width="12.453125" customWidth="1"/>
+    <col min="3331" max="3335" width="12.7265625" customWidth="1"/>
+    <col min="3336" max="3336" width="12.90625" customWidth="1"/>
+    <col min="3337" max="3338" width="12.7265625" customWidth="1"/>
+    <col min="3339" max="3342" width="12.90625" customWidth="1"/>
+    <col min="3343" max="3346" width="12.7265625" customWidth="1"/>
+    <col min="3585" max="3585" width="21.08984375" customWidth="1"/>
+    <col min="3586" max="3586" width="12.453125" customWidth="1"/>
+    <col min="3587" max="3591" width="12.7265625" customWidth="1"/>
+    <col min="3592" max="3592" width="12.90625" customWidth="1"/>
+    <col min="3593" max="3594" width="12.7265625" customWidth="1"/>
+    <col min="3595" max="3598" width="12.90625" customWidth="1"/>
+    <col min="3599" max="3602" width="12.7265625" customWidth="1"/>
+    <col min="3841" max="3841" width="21.08984375" customWidth="1"/>
+    <col min="3842" max="3842" width="12.453125" customWidth="1"/>
+    <col min="3843" max="3847" width="12.7265625" customWidth="1"/>
+    <col min="3848" max="3848" width="12.90625" customWidth="1"/>
+    <col min="3849" max="3850" width="12.7265625" customWidth="1"/>
+    <col min="3851" max="3854" width="12.90625" customWidth="1"/>
+    <col min="3855" max="3858" width="12.7265625" customWidth="1"/>
+    <col min="4097" max="4097" width="21.08984375" customWidth="1"/>
+    <col min="4098" max="4098" width="12.453125" customWidth="1"/>
+    <col min="4099" max="4103" width="12.7265625" customWidth="1"/>
+    <col min="4104" max="4104" width="12.90625" customWidth="1"/>
+    <col min="4105" max="4106" width="12.7265625" customWidth="1"/>
+    <col min="4107" max="4110" width="12.90625" customWidth="1"/>
+    <col min="4111" max="4114" width="12.7265625" customWidth="1"/>
+    <col min="4353" max="4353" width="21.08984375" customWidth="1"/>
+    <col min="4354" max="4354" width="12.453125" customWidth="1"/>
+    <col min="4355" max="4359" width="12.7265625" customWidth="1"/>
+    <col min="4360" max="4360" width="12.90625" customWidth="1"/>
+    <col min="4361" max="4362" width="12.7265625" customWidth="1"/>
+    <col min="4363" max="4366" width="12.90625" customWidth="1"/>
+    <col min="4367" max="4370" width="12.7265625" customWidth="1"/>
+    <col min="4609" max="4609" width="21.08984375" customWidth="1"/>
+    <col min="4610" max="4610" width="12.453125" customWidth="1"/>
+    <col min="4611" max="4615" width="12.7265625" customWidth="1"/>
+    <col min="4616" max="4616" width="12.90625" customWidth="1"/>
+    <col min="4617" max="4618" width="12.7265625" customWidth="1"/>
+    <col min="4619" max="4622" width="12.90625" customWidth="1"/>
+    <col min="4623" max="4626" width="12.7265625" customWidth="1"/>
+    <col min="4865" max="4865" width="21.08984375" customWidth="1"/>
+    <col min="4866" max="4866" width="12.453125" customWidth="1"/>
+    <col min="4867" max="4871" width="12.7265625" customWidth="1"/>
+    <col min="4872" max="4872" width="12.90625" customWidth="1"/>
+    <col min="4873" max="4874" width="12.7265625" customWidth="1"/>
+    <col min="4875" max="4878" width="12.90625" customWidth="1"/>
+    <col min="4879" max="4882" width="12.7265625" customWidth="1"/>
+    <col min="5121" max="5121" width="21.08984375" customWidth="1"/>
+    <col min="5122" max="5122" width="12.453125" customWidth="1"/>
+    <col min="5123" max="5127" width="12.7265625" customWidth="1"/>
+    <col min="5128" max="5128" width="12.90625" customWidth="1"/>
+    <col min="5129" max="5130" width="12.7265625" customWidth="1"/>
+    <col min="5131" max="5134" width="12.90625" customWidth="1"/>
+    <col min="5135" max="5138" width="12.7265625" customWidth="1"/>
+    <col min="5377" max="5377" width="21.08984375" customWidth="1"/>
+    <col min="5378" max="5378" width="12.453125" customWidth="1"/>
+    <col min="5379" max="5383" width="12.7265625" customWidth="1"/>
+    <col min="5384" max="5384" width="12.90625" customWidth="1"/>
+    <col min="5385" max="5386" width="12.7265625" customWidth="1"/>
+    <col min="5387" max="5390" width="12.90625" customWidth="1"/>
+    <col min="5391" max="5394" width="12.7265625" customWidth="1"/>
+    <col min="5633" max="5633" width="21.08984375" customWidth="1"/>
+    <col min="5634" max="5634" width="12.453125" customWidth="1"/>
+    <col min="5635" max="5639" width="12.7265625" customWidth="1"/>
+    <col min="5640" max="5640" width="12.90625" customWidth="1"/>
+    <col min="5641" max="5642" width="12.7265625" customWidth="1"/>
+    <col min="5643" max="5646" width="12.90625" customWidth="1"/>
+    <col min="5647" max="5650" width="12.7265625" customWidth="1"/>
+    <col min="5889" max="5889" width="21.08984375" customWidth="1"/>
+    <col min="5890" max="5890" width="12.453125" customWidth="1"/>
+    <col min="5891" max="5895" width="12.7265625" customWidth="1"/>
+    <col min="5896" max="5896" width="12.90625" customWidth="1"/>
+    <col min="5897" max="5898" width="12.7265625" customWidth="1"/>
+    <col min="5899" max="5902" width="12.90625" customWidth="1"/>
+    <col min="5903" max="5906" width="12.7265625" customWidth="1"/>
+    <col min="6145" max="6145" width="21.08984375" customWidth="1"/>
+    <col min="6146" max="6146" width="12.453125" customWidth="1"/>
+    <col min="6147" max="6151" width="12.7265625" customWidth="1"/>
+    <col min="6152" max="6152" width="12.90625" customWidth="1"/>
+    <col min="6153" max="6154" width="12.7265625" customWidth="1"/>
+    <col min="6155" max="6158" width="12.90625" customWidth="1"/>
+    <col min="6159" max="6162" width="12.7265625" customWidth="1"/>
+    <col min="6401" max="6401" width="21.08984375" customWidth="1"/>
+    <col min="6402" max="6402" width="12.453125" customWidth="1"/>
+    <col min="6403" max="6407" width="12.7265625" customWidth="1"/>
+    <col min="6408" max="6408" width="12.90625" customWidth="1"/>
+    <col min="6409" max="6410" width="12.7265625" customWidth="1"/>
+    <col min="6411" max="6414" width="12.90625" customWidth="1"/>
+    <col min="6415" max="6418" width="12.7265625" customWidth="1"/>
+    <col min="6657" max="6657" width="21.08984375" customWidth="1"/>
+    <col min="6658" max="6658" width="12.453125" customWidth="1"/>
+    <col min="6659" max="6663" width="12.7265625" customWidth="1"/>
+    <col min="6664" max="6664" width="12.90625" customWidth="1"/>
+    <col min="6665" max="6666" width="12.7265625" customWidth="1"/>
+    <col min="6667" max="6670" width="12.90625" customWidth="1"/>
+    <col min="6671" max="6674" width="12.7265625" customWidth="1"/>
+    <col min="6913" max="6913" width="21.08984375" customWidth="1"/>
+    <col min="6914" max="6914" width="12.453125" customWidth="1"/>
+    <col min="6915" max="6919" width="12.7265625" customWidth="1"/>
+    <col min="6920" max="6920" width="12.90625" customWidth="1"/>
+    <col min="6921" max="6922" width="12.7265625" customWidth="1"/>
+    <col min="6923" max="6926" width="12.90625" customWidth="1"/>
+    <col min="6927" max="6930" width="12.7265625" customWidth="1"/>
+    <col min="7169" max="7169" width="21.08984375" customWidth="1"/>
+    <col min="7170" max="7170" width="12.453125" customWidth="1"/>
+    <col min="7171" max="7175" width="12.7265625" customWidth="1"/>
+    <col min="7176" max="7176" width="12.90625" customWidth="1"/>
+    <col min="7177" max="7178" width="12.7265625" customWidth="1"/>
+    <col min="7179" max="7182" width="12.90625" customWidth="1"/>
+    <col min="7183" max="7186" width="12.7265625" customWidth="1"/>
+    <col min="7425" max="7425" width="21.08984375" customWidth="1"/>
+    <col min="7426" max="7426" width="12.453125" customWidth="1"/>
+    <col min="7427" max="7431" width="12.7265625" customWidth="1"/>
+    <col min="7432" max="7432" width="12.90625" customWidth="1"/>
+    <col min="7433" max="7434" width="12.7265625" customWidth="1"/>
+    <col min="7435" max="7438" width="12.90625" customWidth="1"/>
+    <col min="7439" max="7442" width="12.7265625" customWidth="1"/>
+    <col min="7681" max="7681" width="21.08984375" customWidth="1"/>
+    <col min="7682" max="7682" width="12.453125" customWidth="1"/>
+    <col min="7683" max="7687" width="12.7265625" customWidth="1"/>
+    <col min="7688" max="7688" width="12.90625" customWidth="1"/>
+    <col min="7689" max="7690" width="12.7265625" customWidth="1"/>
+    <col min="7691" max="7694" width="12.90625" customWidth="1"/>
+    <col min="7695" max="7698" width="12.7265625" customWidth="1"/>
+    <col min="7937" max="7937" width="21.08984375" customWidth="1"/>
+    <col min="7938" max="7938" width="12.453125" customWidth="1"/>
+    <col min="7939" max="7943" width="12.7265625" customWidth="1"/>
+    <col min="7944" max="7944" width="12.90625" customWidth="1"/>
+    <col min="7945" max="7946" width="12.7265625" customWidth="1"/>
+    <col min="7947" max="7950" width="12.90625" customWidth="1"/>
+    <col min="7951" max="7954" width="12.7265625" customWidth="1"/>
+    <col min="8193" max="8193" width="21.08984375" customWidth="1"/>
+    <col min="8194" max="8194" width="12.453125" customWidth="1"/>
+    <col min="8195" max="8199" width="12.7265625" customWidth="1"/>
+    <col min="8200" max="8200" width="12.90625" customWidth="1"/>
+    <col min="8201" max="8202" width="12.7265625" customWidth="1"/>
+    <col min="8203" max="8206" width="12.90625" customWidth="1"/>
+    <col min="8207" max="8210" width="12.7265625" customWidth="1"/>
+    <col min="8449" max="8449" width="21.08984375" customWidth="1"/>
+    <col min="8450" max="8450" width="12.453125" customWidth="1"/>
+    <col min="8451" max="8455" width="12.7265625" customWidth="1"/>
+    <col min="8456" max="8456" width="12.90625" customWidth="1"/>
+    <col min="8457" max="8458" width="12.7265625" customWidth="1"/>
+    <col min="8459" max="8462" width="12.90625" customWidth="1"/>
+    <col min="8463" max="8466" width="12.7265625" customWidth="1"/>
+    <col min="8705" max="8705" width="21.08984375" customWidth="1"/>
+    <col min="8706" max="8706" width="12.453125" customWidth="1"/>
+    <col min="8707" max="8711" width="12.7265625" customWidth="1"/>
+    <col min="8712" max="8712" width="12.90625" customWidth="1"/>
+    <col min="8713" max="8714" width="12.7265625" customWidth="1"/>
+    <col min="8715" max="8718" width="12.90625" customWidth="1"/>
+    <col min="8719" max="8722" width="12.7265625" customWidth="1"/>
+    <col min="8961" max="8961" width="21.08984375" customWidth="1"/>
+    <col min="8962" max="8962" width="12.453125" customWidth="1"/>
+    <col min="8963" max="8967" width="12.7265625" customWidth="1"/>
+    <col min="8968" max="8968" width="12.90625" customWidth="1"/>
+    <col min="8969" max="8970" width="12.7265625" customWidth="1"/>
+    <col min="8971" max="8974" width="12.90625" customWidth="1"/>
+    <col min="8975" max="8978" width="12.7265625" customWidth="1"/>
+    <col min="9217" max="9217" width="21.08984375" customWidth="1"/>
+    <col min="9218" max="9218" width="12.453125" customWidth="1"/>
+    <col min="9219" max="9223" width="12.7265625" customWidth="1"/>
+    <col min="9224" max="9224" width="12.90625" customWidth="1"/>
+    <col min="9225" max="9226" width="12.7265625" customWidth="1"/>
+    <col min="9227" max="9230" width="12.90625" customWidth="1"/>
+    <col min="9231" max="9234" width="12.7265625" customWidth="1"/>
+    <col min="9473" max="9473" width="21.08984375" customWidth="1"/>
+    <col min="9474" max="9474" width="12.453125" customWidth="1"/>
+    <col min="9475" max="9479" width="12.7265625" customWidth="1"/>
+    <col min="9480" max="9480" width="12.90625" customWidth="1"/>
+    <col min="9481" max="9482" width="12.7265625" customWidth="1"/>
+    <col min="9483" max="9486" width="12.90625" customWidth="1"/>
+    <col min="9487" max="9490" width="12.7265625" customWidth="1"/>
+    <col min="9729" max="9729" width="21.08984375" customWidth="1"/>
+    <col min="9730" max="9730" width="12.453125" customWidth="1"/>
+    <col min="9731" max="9735" width="12.7265625" customWidth="1"/>
+    <col min="9736" max="9736" width="12.90625" customWidth="1"/>
+    <col min="9737" max="9738" width="12.7265625" customWidth="1"/>
+    <col min="9739" max="9742" width="12.90625" customWidth="1"/>
+    <col min="9743" max="9746" width="12.7265625" customWidth="1"/>
+    <col min="9985" max="9985" width="21.08984375" customWidth="1"/>
+    <col min="9986" max="9986" width="12.453125" customWidth="1"/>
+    <col min="9987" max="9991" width="12.7265625" customWidth="1"/>
+    <col min="9992" max="9992" width="12.90625" customWidth="1"/>
+    <col min="9993" max="9994" width="12.7265625" customWidth="1"/>
+    <col min="9995" max="9998" width="12.90625" customWidth="1"/>
+    <col min="9999" max="10002" width="12.7265625" customWidth="1"/>
+    <col min="10241" max="10241" width="21.08984375" customWidth="1"/>
+    <col min="10242" max="10242" width="12.453125" customWidth="1"/>
+    <col min="10243" max="10247" width="12.7265625" customWidth="1"/>
+    <col min="10248" max="10248" width="12.90625" customWidth="1"/>
+    <col min="10249" max="10250" width="12.7265625" customWidth="1"/>
+    <col min="10251" max="10254" width="12.90625" customWidth="1"/>
+    <col min="10255" max="10258" width="12.7265625" customWidth="1"/>
+    <col min="10497" max="10497" width="21.08984375" customWidth="1"/>
+    <col min="10498" max="10498" width="12.453125" customWidth="1"/>
+    <col min="10499" max="10503" width="12.7265625" customWidth="1"/>
+    <col min="10504" max="10504" width="12.90625" customWidth="1"/>
+    <col min="10505" max="10506" width="12.7265625" customWidth="1"/>
+    <col min="10507" max="10510" width="12.90625" customWidth="1"/>
+    <col min="10511" max="10514" width="12.7265625" customWidth="1"/>
+    <col min="10753" max="10753" width="21.08984375" customWidth="1"/>
+    <col min="10754" max="10754" width="12.453125" customWidth="1"/>
+    <col min="10755" max="10759" width="12.7265625" customWidth="1"/>
+    <col min="10760" max="10760" width="12.90625" customWidth="1"/>
+    <col min="10761" max="10762" width="12.7265625" customWidth="1"/>
+    <col min="10763" max="10766" width="12.90625" customWidth="1"/>
+    <col min="10767" max="10770" width="12.7265625" customWidth="1"/>
+    <col min="11009" max="11009" width="21.08984375" customWidth="1"/>
+    <col min="11010" max="11010" width="12.453125" customWidth="1"/>
+    <col min="11011" max="11015" width="12.7265625" customWidth="1"/>
+    <col min="11016" max="11016" width="12.90625" customWidth="1"/>
+    <col min="11017" max="11018" width="12.7265625" customWidth="1"/>
+    <col min="11019" max="11022" width="12.90625" customWidth="1"/>
+    <col min="11023" max="11026" width="12.7265625" customWidth="1"/>
+    <col min="11265" max="11265" width="21.08984375" customWidth="1"/>
+    <col min="11266" max="11266" width="12.453125" customWidth="1"/>
+    <col min="11267" max="11271" width="12.7265625" customWidth="1"/>
+    <col min="11272" max="11272" width="12.90625" customWidth="1"/>
+    <col min="11273" max="11274" width="12.7265625" customWidth="1"/>
+    <col min="11275" max="11278" width="12.90625" customWidth="1"/>
+    <col min="11279" max="11282" width="12.7265625" customWidth="1"/>
+    <col min="11521" max="11521" width="21.08984375" customWidth="1"/>
+    <col min="11522" max="11522" width="12.453125" customWidth="1"/>
+    <col min="11523" max="11527" width="12.7265625" customWidth="1"/>
+    <col min="11528" max="11528" width="12.90625" customWidth="1"/>
+    <col min="11529" max="11530" width="12.7265625" customWidth="1"/>
+    <col min="11531" max="11534" width="12.90625" customWidth="1"/>
+    <col min="11535" max="11538" width="12.7265625" customWidth="1"/>
+    <col min="11777" max="11777" width="21.08984375" customWidth="1"/>
+    <col min="11778" max="11778" width="12.453125" customWidth="1"/>
+    <col min="11779" max="11783" width="12.7265625" customWidth="1"/>
+    <col min="11784" max="11784" width="12.90625" customWidth="1"/>
+    <col min="11785" max="11786" width="12.7265625" customWidth="1"/>
+    <col min="11787" max="11790" width="12.90625" customWidth="1"/>
+    <col min="11791" max="11794" width="12.7265625" customWidth="1"/>
+    <col min="12033" max="12033" width="21.08984375" customWidth="1"/>
+    <col min="12034" max="12034" width="12.453125" customWidth="1"/>
+    <col min="12035" max="12039" width="12.7265625" customWidth="1"/>
+    <col min="12040" max="12040" width="12.90625" customWidth="1"/>
+    <col min="12041" max="12042" width="12.7265625" customWidth="1"/>
+    <col min="12043" max="12046" width="12.90625" customWidth="1"/>
+    <col min="12047" max="12050" width="12.7265625" customWidth="1"/>
+    <col min="12289" max="12289" width="21.08984375" customWidth="1"/>
+    <col min="12290" max="12290" width="12.453125" customWidth="1"/>
+    <col min="12291" max="12295" width="12.7265625" customWidth="1"/>
+    <col min="12296" max="12296" width="12.90625" customWidth="1"/>
+    <col min="12297" max="12298" width="12.7265625" customWidth="1"/>
+    <col min="12299" max="12302" width="12.90625" customWidth="1"/>
+    <col min="12303" max="12306" width="12.7265625" customWidth="1"/>
+    <col min="12545" max="12545" width="21.08984375" customWidth="1"/>
+    <col min="12546" max="12546" width="12.453125" customWidth="1"/>
+    <col min="12547" max="12551" width="12.7265625" customWidth="1"/>
+    <col min="12552" max="12552" width="12.90625" customWidth="1"/>
+    <col min="12553" max="12554" width="12.7265625" customWidth="1"/>
+    <col min="12555" max="12558" width="12.90625" customWidth="1"/>
+    <col min="12559" max="12562" width="12.7265625" customWidth="1"/>
+    <col min="12801" max="12801" width="21.08984375" customWidth="1"/>
+    <col min="12802" max="12802" width="12.453125" customWidth="1"/>
+    <col min="12803" max="12807" width="12.7265625" customWidth="1"/>
+    <col min="12808" max="12808" width="12.90625" customWidth="1"/>
+    <col min="12809" max="12810" width="12.7265625" customWidth="1"/>
+    <col min="12811" max="12814" width="12.90625" customWidth="1"/>
+    <col min="12815" max="12818" width="12.7265625" customWidth="1"/>
+    <col min="13057" max="13057" width="21.08984375" customWidth="1"/>
+    <col min="13058" max="13058" width="12.453125" customWidth="1"/>
+    <col min="13059" max="13063" width="12.7265625" customWidth="1"/>
+    <col min="13064" max="13064" width="12.90625" customWidth="1"/>
+    <col min="13065" max="13066" width="12.7265625" customWidth="1"/>
+    <col min="13067" max="13070" width="12.90625" customWidth="1"/>
+    <col min="13071" max="13074" width="12.7265625" customWidth="1"/>
+    <col min="13313" max="13313" width="21.08984375" customWidth="1"/>
+    <col min="13314" max="13314" width="12.453125" customWidth="1"/>
+    <col min="13315" max="13319" width="12.7265625" customWidth="1"/>
+    <col min="13320" max="13320" width="12.90625" customWidth="1"/>
+    <col min="13321" max="13322" width="12.7265625" customWidth="1"/>
+    <col min="13323" max="13326" width="12.90625" customWidth="1"/>
+    <col min="13327" max="13330" width="12.7265625" customWidth="1"/>
+    <col min="13569" max="13569" width="21.08984375" customWidth="1"/>
+    <col min="13570" max="13570" width="12.453125" customWidth="1"/>
+    <col min="13571" max="13575" width="12.7265625" customWidth="1"/>
+    <col min="13576" max="13576" width="12.90625" customWidth="1"/>
+    <col min="13577" max="13578" width="12.7265625" customWidth="1"/>
+    <col min="13579" max="13582" width="12.90625" customWidth="1"/>
+    <col min="13583" max="13586" width="12.7265625" customWidth="1"/>
+    <col min="13825" max="13825" width="21.08984375" customWidth="1"/>
+    <col min="13826" max="13826" width="12.453125" customWidth="1"/>
+    <col min="13827" max="13831" width="12.7265625" customWidth="1"/>
+    <col min="13832" max="13832" width="12.90625" customWidth="1"/>
+    <col min="13833" max="13834" width="12.7265625" customWidth="1"/>
+    <col min="13835" max="13838" width="12.90625" customWidth="1"/>
+    <col min="13839" max="13842" width="12.7265625" customWidth="1"/>
+    <col min="14081" max="14081" width="21.08984375" customWidth="1"/>
+    <col min="14082" max="14082" width="12.453125" customWidth="1"/>
+    <col min="14083" max="14087" width="12.7265625" customWidth="1"/>
+    <col min="14088" max="14088" width="12.90625" customWidth="1"/>
+    <col min="14089" max="14090" width="12.7265625" customWidth="1"/>
+    <col min="14091" max="14094" width="12.90625" customWidth="1"/>
+    <col min="14095" max="14098" width="12.7265625" customWidth="1"/>
+    <col min="14337" max="14337" width="21.08984375" customWidth="1"/>
+    <col min="14338" max="14338" width="12.453125" customWidth="1"/>
+    <col min="14339" max="14343" width="12.7265625" customWidth="1"/>
+    <col min="14344" max="14344" width="12.90625" customWidth="1"/>
+    <col min="14345" max="14346" width="12.7265625" customWidth="1"/>
+    <col min="14347" max="14350" width="12.90625" customWidth="1"/>
+    <col min="14351" max="14354" width="12.7265625" customWidth="1"/>
+    <col min="14593" max="14593" width="21.08984375" customWidth="1"/>
+    <col min="14594" max="14594" width="12.453125" customWidth="1"/>
+    <col min="14595" max="14599" width="12.7265625" customWidth="1"/>
+    <col min="14600" max="14600" width="12.90625" customWidth="1"/>
+    <col min="14601" max="14602" width="12.7265625" customWidth="1"/>
+    <col min="14603" max="14606" width="12.90625" customWidth="1"/>
+    <col min="14607" max="14610" width="12.7265625" customWidth="1"/>
+    <col min="14849" max="14849" width="21.08984375" customWidth="1"/>
+    <col min="14850" max="14850" width="12.453125" customWidth="1"/>
+    <col min="14851" max="14855" width="12.7265625" customWidth="1"/>
+    <col min="14856" max="14856" width="12.90625" customWidth="1"/>
+    <col min="14857" max="14858" width="12.7265625" customWidth="1"/>
+    <col min="14859" max="14862" width="12.90625" customWidth="1"/>
+    <col min="14863" max="14866" width="12.7265625" customWidth="1"/>
+    <col min="15105" max="15105" width="21.08984375" customWidth="1"/>
+    <col min="15106" max="15106" width="12.453125" customWidth="1"/>
+    <col min="15107" max="15111" width="12.7265625" customWidth="1"/>
+    <col min="15112" max="15112" width="12.90625" customWidth="1"/>
+    <col min="15113" max="15114" width="12.7265625" customWidth="1"/>
+    <col min="15115" max="15118" width="12.90625" customWidth="1"/>
+    <col min="15119" max="15122" width="12.7265625" customWidth="1"/>
+    <col min="15361" max="15361" width="21.08984375" customWidth="1"/>
+    <col min="15362" max="15362" width="12.453125" customWidth="1"/>
+    <col min="15363" max="15367" width="12.7265625" customWidth="1"/>
+    <col min="15368" max="15368" width="12.90625" customWidth="1"/>
+    <col min="15369" max="15370" width="12.7265625" customWidth="1"/>
+    <col min="15371" max="15374" width="12.90625" customWidth="1"/>
+    <col min="15375" max="15378" width="12.7265625" customWidth="1"/>
+    <col min="15617" max="15617" width="21.08984375" customWidth="1"/>
+    <col min="15618" max="15618" width="12.453125" customWidth="1"/>
+    <col min="15619" max="15623" width="12.7265625" customWidth="1"/>
+    <col min="15624" max="15624" width="12.90625" customWidth="1"/>
+    <col min="15625" max="15626" width="12.7265625" customWidth="1"/>
+    <col min="15627" max="15630" width="12.90625" customWidth="1"/>
+    <col min="15631" max="15634" width="12.7265625" customWidth="1"/>
+    <col min="15873" max="15873" width="21.08984375" customWidth="1"/>
+    <col min="15874" max="15874" width="12.453125" customWidth="1"/>
+    <col min="15875" max="15879" width="12.7265625" customWidth="1"/>
+    <col min="15880" max="15880" width="12.90625" customWidth="1"/>
+    <col min="15881" max="15882" width="12.7265625" customWidth="1"/>
+    <col min="15883" max="15886" width="12.90625" customWidth="1"/>
+    <col min="15887" max="15890" width="12.7265625" customWidth="1"/>
+    <col min="16129" max="16129" width="21.08984375" customWidth="1"/>
+    <col min="16130" max="16130" width="12.453125" customWidth="1"/>
+    <col min="16131" max="16135" width="12.7265625" customWidth="1"/>
+    <col min="16136" max="16136" width="12.90625" customWidth="1"/>
+    <col min="16137" max="16138" width="12.7265625" customWidth="1"/>
+    <col min="16139" max="16142" width="12.90625" customWidth="1"/>
+    <col min="16143" max="16146" width="12.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -26259,6 +26296,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
     <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
@@ -26402,29 +26454,37 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1139C0F6-B00C-4379-81CA-44285F52FF2E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{63D16A6B-8B1B-4121-BE38-0F3E968A7BF0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30D49544-8BCC-440A-9096-15397E5D5534}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30D49544-8BCC-440A-9096-15397E5D5534}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{63D16A6B-8B1B-4121-BE38-0F3E968A7BF0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1139C0F6-B00C-4379-81CA-44285F52FF2E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="40f4d404-d193-41dc-bb72-733c1e774208"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updates aircraft calibration to represent domestic-only flights
</commit_message>
<xml_diff>
--- a/InputData/trans/AVLo/Avg Vehicle Loading.xlsx
+++ b/InputData/trans/AVLo/Avg Vehicle Loading.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\SK\eps-southkorea\InputData\trans\AVLo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD60A80E-C49D-4DF4-920E-4DEF305E23E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4237D3BD-6791-4CBA-BE32-3321F4032A71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5670" yWindow="3225" windowWidth="22005" windowHeight="13365" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28410" yWindow="390" windowWidth="25050" windowHeight="14970" firstSheet="9" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -23,20 +23,27 @@
     <sheet name="subway" sheetId="12" r:id="rId8"/>
     <sheet name="고속철도 여객수송동향" sheetId="14" r:id="rId9"/>
     <sheet name="열차 여객수송인원" sheetId="15" r:id="rId10"/>
-    <sheet name="rail" sheetId="13" r:id="rId11"/>
-    <sheet name="US AVLo" sheetId="17" r:id="rId12"/>
-    <sheet name="SYAVLo-passengers" sheetId="18" r:id="rId13"/>
-    <sheet name="SYAVLo-freight" sheetId="19" r:id="rId14"/>
-    <sheet name="AVLo-passengers" sheetId="2" r:id="rId15"/>
-    <sheet name="AVLo-freight" sheetId="4" r:id="rId16"/>
+    <sheet name="Air-Calcs" sheetId="20" r:id="rId11"/>
+    <sheet name="rail" sheetId="13" r:id="rId12"/>
+    <sheet name="US AVLo" sheetId="17" r:id="rId13"/>
+    <sheet name="SYAVLo-passengers" sheetId="18" r:id="rId14"/>
+    <sheet name="SYAVLo-freight" sheetId="19" r:id="rId15"/>
+    <sheet name="AVLo-passengers" sheetId="2" r:id="rId16"/>
+    <sheet name="AVLo-freight" sheetId="4" r:id="rId17"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId17"/>
+    <externalReference r:id="rId18"/>
+    <externalReference r:id="rId19"/>
+    <externalReference r:id="rId20"/>
   </externalReferences>
   <definedNames>
+    <definedName name="Eno_TM" localSheetId="10">'[3]1997  Table 1a Modified'!#REF!</definedName>
     <definedName name="Eno_TM">'[1]1997  Table 1a Modified'!#REF!</definedName>
+    <definedName name="Eno_Tons" localSheetId="10">'[3]1997  Table 1a Modified'!#REF!</definedName>
     <definedName name="Eno_Tons">'[1]1997  Table 1a Modified'!#REF!</definedName>
+    <definedName name="Sum_T2" localSheetId="10">'[3]1997  Table 1a Modified'!#REF!</definedName>
     <definedName name="Sum_T2">'[1]1997  Table 1a Modified'!#REF!</definedName>
+    <definedName name="Sum_TTM" localSheetId="10">'[3]1997  Table 1a Modified'!#REF!</definedName>
     <definedName name="Sum_TTM">'[1]1997  Table 1a Modified'!#REF!</definedName>
     <definedName name="ti_tbl_50">#REF!</definedName>
     <definedName name="ti_tbl_69">#REF!</definedName>
@@ -57,8 +64,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="497">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="519">
   <si>
     <t>AVLo Average Vehicle Loading</t>
   </si>
@@ -1863,6 +1892,95 @@
     <t>In the case of Korean freight ships, most of them are international cargo transport,</t>
     <phoneticPr fontId="42" type="noConversion"/>
   </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>International passengers</t>
+  </si>
+  <si>
+    <t>Domestic passengers</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>pgs. 22-23, 16-17, 18-19</t>
+  </si>
+  <si>
+    <t>psgr-mi</t>
+  </si>
+  <si>
+    <t>pkt</t>
+  </si>
+  <si>
+    <t>km/flight</t>
+  </si>
+  <si>
+    <t>Non-scheduled</t>
+  </si>
+  <si>
+    <t>Scheduled</t>
+  </si>
+  <si>
+    <t>Flight Kilometers (Total)</t>
+  </si>
+  <si>
+    <t>Flights (Total)</t>
+  </si>
+  <si>
+    <t>1-6. Domestic Flight Operation Performance</t>
+  </si>
+  <si>
+    <t>pg. 56</t>
+  </si>
+  <si>
+    <t>pg. 16</t>
+  </si>
+  <si>
+    <t>passengers</t>
+  </si>
+  <si>
+    <t>32.98 (2019) → 25.16 (2020) → 33.15 (2021) → 36.33 (2022) → 32.19 (2023) → 31.13 (2024)</t>
+  </si>
+  <si>
+    <t>Domestic passengers (10,000 persons):</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">In 2024, domestic air passengers decreased due to a continued rise in overseas travel demand, which led to reduced domestic flight operations. Both Jeju and inland routes saw declines, resulting in a 3.3% drop year-over-year to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>31.13 million passengers</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>A. Overview</t>
+  </si>
+  <si>
+    <t>p. 32</t>
+  </si>
+  <si>
+    <t>https://www.airportal.go.kr/file/htmlOpen/upload/ebook/Stats2025/</t>
+  </si>
 </sst>
 </file>
 
@@ -1880,7 +1998,7 @@
     <numFmt numFmtId="170" formatCode="0.0_ "/>
     <numFmt numFmtId="171" formatCode="0_ "/>
   </numFmts>
-  <fonts count="60">
+  <fonts count="61">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2255,6 +2373,14 @@
       <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -3259,7 +3385,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="131">
+  <cellXfs count="139">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -3571,6 +3697,26 @@
     <xf numFmtId="0" fontId="41" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="155">
     <cellStyle name="20% - Accent1 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -3974,6 +4120,50 @@
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="4599061" cy="3448050"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8202BD6F-F88D-4DE6-8526-28F8B49F62F8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="381000"/>
+          <a:ext cx="4599061" cy="3448050"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -4024,6 +4214,183 @@
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="Rail shipments 93-97"/>
+      <sheetName val="Waterborne Flows 93-97"/>
+      <sheetName val="Air and vessel 93-97"/>
+      <sheetName val="Figure 2 compare"/>
+      <sheetName val="Factors Comparisons"/>
+      <sheetName val="1997  Table 1a Modified"/>
+      <sheetName val="Figure 1"/>
+      <sheetName val="1993-97 Table 1  US Highlights"/>
+      <sheetName val="93-97 US Freight Table 1"/>
+      <sheetName val="93-97 US Freight Table 1 (b)"/>
+      <sheetName val="93-97 Percents Tab 2&amp;3"/>
+      <sheetName val="Integrated View 93-97"/>
+      <sheetName val="Figure 3 modal shares"/>
+      <sheetName val="1993-97 Percents"/>
+      <sheetName val="BTS &amp; ORNL estimates"/>
+      <sheetName val="Oil Pipeline (2)"/>
+      <sheetName val="1997 Table 2"/>
+      <sheetName val="Table 4 Distance"/>
+      <sheetName val="Distance percent change"/>
+      <sheetName val="Distance 93-97"/>
+      <sheetName val="Distance Fig value per ton"/>
+      <sheetName val="Distance Bar"/>
+      <sheetName val="Table 5 Size 93-97"/>
+      <sheetName val="Size percent change"/>
+      <sheetName val="Size Fig value per ton"/>
+      <sheetName val="Size Bar "/>
+      <sheetName val="BTS Mode"/>
+      <sheetName val="Ton-miles data"/>
+      <sheetName val="Ton-miles figure"/>
+      <sheetName val="table 3 commodities"/>
+      <sheetName val="Commodities ranked by value"/>
+      <sheetName val="Commod ranked by tons"/>
+      <sheetName val="Commod ranked by ton-miles"/>
+      <sheetName val="Commod ranked by miles per ton "/>
+      <sheetName val="Commod ranked by val per ton"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
+      <sheetData sheetId="14"/>
+      <sheetData sheetId="15"/>
+      <sheetData sheetId="16"/>
+      <sheetData sheetId="17"/>
+      <sheetData sheetId="18"/>
+      <sheetData sheetId="19"/>
+      <sheetData sheetId="20"/>
+      <sheetData sheetId="21" refreshError="1"/>
+      <sheetData sheetId="22"/>
+      <sheetData sheetId="23"/>
+      <sheetData sheetId="24"/>
+      <sheetData sheetId="25" refreshError="1"/>
+      <sheetData sheetId="26"/>
+      <sheetData sheetId="27"/>
+      <sheetData sheetId="28"/>
+      <sheetData sheetId="29"/>
+      <sheetData sheetId="30"/>
+      <sheetData sheetId="31"/>
+      <sheetData sheetId="32"/>
+      <sheetData sheetId="33"/>
+      <sheetData sheetId="34"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="About"/>
+      <sheetName val="SYVbT_passenger"/>
+      <sheetName val="SYVbT_freight"/>
+      <sheetName val="SYVbT_DV-Regis"/>
+      <sheetName val="DV-km"/>
+      <sheetName val="DV-Cal"/>
+      <sheetName val="SYVbT_Rail"/>
+      <sheetName val="Rail-domestic psgr traffic"/>
+      <sheetName val="Rail-CAGR"/>
+      <sheetName val="Rail-subway"/>
+      <sheetName val="Rail-Cal"/>
+      <sheetName val="SYVbT_Aircraft"/>
+      <sheetName val="Air09"/>
+      <sheetName val="Air10"/>
+      <sheetName val="Air11"/>
+      <sheetName val="Air12"/>
+      <sheetName val="Air13"/>
+      <sheetName val="Air14"/>
+      <sheetName val="Air15"/>
+      <sheetName val="Air16"/>
+      <sheetName val="Air17"/>
+      <sheetName val="Air18"/>
+      <sheetName val="Air19"/>
+      <sheetName val="Air20"/>
+      <sheetName val="Air21"/>
+      <sheetName val="Air-psgr19"/>
+      <sheetName val="Air-freight19"/>
+      <sheetName val="Air-Cal"/>
+      <sheetName val="Motorbikes"/>
+      <sheetName val="Ships-Cal"/>
+      <sheetName val="SYAADTbVT-passengers"/>
+      <sheetName val="SYAADTbVT-freight"/>
+      <sheetName val="BAADTbVT-passengers"/>
+      <sheetName val="BAADTbVT-freight"/>
+      <sheetName val="AVLo-passenger"/>
+      <sheetName val="AVLo-freight"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="64">
+          <cell r="B64">
+            <v>0.62137100000000001</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
+      <sheetData sheetId="14"/>
+      <sheetData sheetId="15"/>
+      <sheetData sheetId="16"/>
+      <sheetData sheetId="17"/>
+      <sheetData sheetId="18"/>
+      <sheetData sheetId="19"/>
+      <sheetData sheetId="20"/>
+      <sheetData sheetId="21"/>
+      <sheetData sheetId="22"/>
+      <sheetData sheetId="23"/>
+      <sheetData sheetId="24"/>
+      <sheetData sheetId="25"/>
+      <sheetData sheetId="26"/>
+      <sheetData sheetId="27"/>
+      <sheetData sheetId="28"/>
+      <sheetData sheetId="29"/>
+      <sheetData sheetId="30"/>
+      <sheetData sheetId="31"/>
+      <sheetData sheetId="32"/>
+      <sheetData sheetId="33"/>
+      <sheetData sheetId="34"/>
+      <sheetData sheetId="35"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Rail shipments 93-97"/>
       <sheetName val="Waterborne Flows 93-97"/>
@@ -5669,6 +6036,714 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39261612-B7A0-4B40-8A97-686A4FA3FEBF}">
+  <dimension ref="A1:M60"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="2" width="10.85546875" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" customWidth="1"/>
+    <col min="4" max="7" width="10.85546875" customWidth="1"/>
+    <col min="10" max="10" width="15.42578125" customWidth="1"/>
+    <col min="11" max="11" width="14.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" s="1" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" s="137"/>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" s="137" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" s="137" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="B28" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29">
+        <v>2019</v>
+      </c>
+      <c r="B29">
+        <v>32980000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30">
+        <v>2020</v>
+      </c>
+      <c r="B30">
+        <v>25160000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31">
+        <v>2021</v>
+      </c>
+      <c r="B31" s="136">
+        <v>33146646</v>
+      </c>
+      <c r="C31" s="136" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32">
+        <v>2022</v>
+      </c>
+      <c r="B32" s="136">
+        <v>36328296</v>
+      </c>
+      <c r="C32" s="136" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13">
+      <c r="A33">
+        <v>2023</v>
+      </c>
+      <c r="B33" s="136">
+        <v>32189676</v>
+      </c>
+      <c r="C33" s="136" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13">
+      <c r="A34">
+        <v>2024</v>
+      </c>
+      <c r="B34" s="136">
+        <v>31131750</v>
+      </c>
+      <c r="C34" s="136" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13">
+      <c r="A36" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13">
+      <c r="A37" s="1" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" ht="45">
+      <c r="A38" s="134" t="s">
+        <v>500</v>
+      </c>
+      <c r="B38" s="134" t="s">
+        <v>508</v>
+      </c>
+      <c r="C38" s="134" t="s">
+        <v>506</v>
+      </c>
+      <c r="D38" s="134" t="s">
+        <v>505</v>
+      </c>
+      <c r="E38" s="134" t="s">
+        <v>507</v>
+      </c>
+      <c r="F38" s="134" t="s">
+        <v>506</v>
+      </c>
+      <c r="G38" s="134" t="s">
+        <v>505</v>
+      </c>
+      <c r="I38" s="1" t="s">
+        <v>504</v>
+      </c>
+      <c r="J38" s="134" t="s">
+        <v>503</v>
+      </c>
+      <c r="K38" s="134" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13">
+      <c r="A39" s="132">
+        <v>2012</v>
+      </c>
+      <c r="B39" s="135">
+        <v>155609</v>
+      </c>
+      <c r="C39" s="135">
+        <v>148765</v>
+      </c>
+      <c r="D39" s="135">
+        <v>6844</v>
+      </c>
+      <c r="E39" s="135">
+        <v>61719336</v>
+      </c>
+      <c r="F39" s="135">
+        <v>58589680</v>
+      </c>
+      <c r="G39" s="135">
+        <v>3129656</v>
+      </c>
+      <c r="I39" s="3">
+        <f>E39/B39</f>
+        <v>396.63088895886483</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13">
+      <c r="A40" s="132">
+        <v>2013</v>
+      </c>
+      <c r="B40" s="135">
+        <v>161750</v>
+      </c>
+      <c r="C40" s="135">
+        <v>155952</v>
+      </c>
+      <c r="D40" s="135">
+        <v>5798</v>
+      </c>
+      <c r="E40" s="135">
+        <v>64559278</v>
+      </c>
+      <c r="F40" s="135">
+        <v>61929709</v>
+      </c>
+      <c r="G40" s="135">
+        <v>2629569</v>
+      </c>
+      <c r="I40" s="3">
+        <f>E40/B40</f>
+        <v>399.13000309119013</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13">
+      <c r="A41" s="132">
+        <v>2014</v>
+      </c>
+      <c r="B41" s="135">
+        <v>170101</v>
+      </c>
+      <c r="C41" s="135">
+        <v>165102</v>
+      </c>
+      <c r="D41" s="135">
+        <v>4999</v>
+      </c>
+      <c r="E41" s="135">
+        <v>63709330</v>
+      </c>
+      <c r="F41" s="135">
+        <v>61583360</v>
+      </c>
+      <c r="G41" s="135">
+        <v>2125970</v>
+      </c>
+      <c r="I41" s="3">
+        <f>E41/B41</f>
+        <v>374.53824492507391</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13">
+      <c r="A42" s="132">
+        <v>2015</v>
+      </c>
+      <c r="B42" s="135">
+        <v>182583</v>
+      </c>
+      <c r="C42" s="135">
+        <v>179336</v>
+      </c>
+      <c r="D42" s="135">
+        <v>3247</v>
+      </c>
+      <c r="E42" s="135">
+        <v>68317092</v>
+      </c>
+      <c r="F42" s="135">
+        <v>67006009</v>
+      </c>
+      <c r="G42" s="135">
+        <v>1311083</v>
+      </c>
+      <c r="I42" s="3">
+        <f>E42/B42</f>
+        <v>374.17005964410708</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13">
+      <c r="A43" s="132">
+        <v>2016</v>
+      </c>
+      <c r="B43" s="135">
+        <v>190997</v>
+      </c>
+      <c r="C43" s="135">
+        <v>188293</v>
+      </c>
+      <c r="D43" s="135">
+        <v>2704</v>
+      </c>
+      <c r="E43" s="135">
+        <v>71694540</v>
+      </c>
+      <c r="F43" s="135">
+        <v>70606148</v>
+      </c>
+      <c r="G43" s="135">
+        <v>1088392</v>
+      </c>
+      <c r="I43" s="3">
+        <f>E43/B43</f>
+        <v>375.36997963318794</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13">
+      <c r="A44" s="132">
+        <v>2017</v>
+      </c>
+      <c r="B44" s="135">
+        <v>196555</v>
+      </c>
+      <c r="C44" s="135">
+        <v>193186</v>
+      </c>
+      <c r="D44" s="135">
+        <v>3369</v>
+      </c>
+      <c r="E44" s="135">
+        <v>72770168</v>
+      </c>
+      <c r="F44" s="135">
+        <v>71446069</v>
+      </c>
+      <c r="G44" s="135">
+        <v>1324099</v>
+      </c>
+      <c r="I44" s="3">
+        <f>E44/B44</f>
+        <v>370.22801760321539</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13">
+      <c r="A45" s="132">
+        <v>2018</v>
+      </c>
+      <c r="B45" s="135">
+        <v>194432</v>
+      </c>
+      <c r="C45" s="135">
+        <v>191135</v>
+      </c>
+      <c r="D45" s="135">
+        <v>3297</v>
+      </c>
+      <c r="E45" s="135">
+        <v>71323490</v>
+      </c>
+      <c r="F45" s="135">
+        <v>70040450</v>
+      </c>
+      <c r="G45" s="135">
+        <v>1283040</v>
+      </c>
+      <c r="I45" s="3">
+        <f>E45/B45</f>
+        <v>366.82999711981569</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13">
+      <c r="A46" s="132">
+        <v>2019</v>
+      </c>
+      <c r="B46" s="135">
+        <v>195349</v>
+      </c>
+      <c r="C46" s="135">
+        <v>190859</v>
+      </c>
+      <c r="D46" s="135">
+        <v>4490</v>
+      </c>
+      <c r="E46" s="135">
+        <v>71936173</v>
+      </c>
+      <c r="F46" s="135">
+        <v>70243770</v>
+      </c>
+      <c r="G46" s="135">
+        <v>1692403</v>
+      </c>
+      <c r="I46" s="3">
+        <f>E46/B46</f>
+        <v>368.24438824872408</v>
+      </c>
+      <c r="J46" s="26">
+        <f>I46*B29</f>
+        <v>12144699924.442921</v>
+      </c>
+      <c r="K46" s="26">
+        <f>J46*[2]About!$B$64</f>
+        <v>7546364336.7510223</v>
+      </c>
+      <c r="M46" s="3">
+        <f>J46/E46</f>
+        <v>168.82604978781566</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13">
+      <c r="A47" s="132">
+        <v>2020</v>
+      </c>
+      <c r="B47" s="135">
+        <v>172383</v>
+      </c>
+      <c r="C47" s="135">
+        <v>149060</v>
+      </c>
+      <c r="D47" s="135">
+        <v>23323</v>
+      </c>
+      <c r="E47" s="135">
+        <v>63640729</v>
+      </c>
+      <c r="F47" s="135">
+        <v>55353366</v>
+      </c>
+      <c r="G47" s="135">
+        <v>8287363</v>
+      </c>
+      <c r="I47" s="3">
+        <f>E47/B47</f>
+        <v>369.18216413451444</v>
+      </c>
+      <c r="J47" s="26">
+        <f>I47*B30</f>
+        <v>9288623249.6243839</v>
+      </c>
+      <c r="K47" s="26">
+        <f>J47*[2]About!$B$64</f>
+        <v>5771681117.2423534</v>
+      </c>
+      <c r="M47" s="3">
+        <f t="shared" ref="M47:M51" si="0">J47/E47</f>
+        <v>145.95406739643701</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13">
+      <c r="A48" s="132">
+        <v>2021</v>
+      </c>
+      <c r="B48" s="135">
+        <v>212690</v>
+      </c>
+      <c r="C48" s="135">
+        <v>195596</v>
+      </c>
+      <c r="D48" s="135">
+        <v>17094</v>
+      </c>
+      <c r="E48" s="135">
+        <v>78207246</v>
+      </c>
+      <c r="F48" s="135">
+        <v>72155503</v>
+      </c>
+      <c r="G48" s="135">
+        <v>6051743</v>
+      </c>
+      <c r="I48" s="3">
+        <f>E48/B48</f>
+        <v>367.70532700173965</v>
+      </c>
+      <c r="J48" s="26">
+        <f>I48*B31</f>
+        <v>12188198306.440905</v>
+      </c>
+      <c r="K48" s="26">
+        <f>J48*[2]About!$B$64</f>
+        <v>7573392969.8714914</v>
+      </c>
+      <c r="M48" s="3">
+        <f t="shared" si="0"/>
+        <v>155.84487281959659</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13">
+      <c r="A49" s="132">
+        <v>2022</v>
+      </c>
+      <c r="B49" s="135">
+        <v>216445</v>
+      </c>
+      <c r="C49" s="135">
+        <v>204195</v>
+      </c>
+      <c r="D49" s="135">
+        <v>12250</v>
+      </c>
+      <c r="E49" s="135">
+        <v>80598677</v>
+      </c>
+      <c r="F49" s="135">
+        <v>75693271</v>
+      </c>
+      <c r="G49" s="135">
+        <v>4905406</v>
+      </c>
+      <c r="I49" s="3">
+        <f>E49/B49</f>
+        <v>372.3748619741736</v>
+      </c>
+      <c r="J49" s="26">
+        <f>I49*B32</f>
+        <v>13527744208.756924</v>
+      </c>
+      <c r="K49" s="26">
+        <f>J49*[2]About!$B$64</f>
+        <v>8405747946.7394981</v>
+      </c>
+      <c r="M49" s="3">
+        <f t="shared" si="0"/>
+        <v>167.84077248261684</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13">
+      <c r="A50" s="132">
+        <v>2023</v>
+      </c>
+      <c r="B50" s="135">
+        <v>191064</v>
+      </c>
+      <c r="C50" s="135">
+        <v>187105</v>
+      </c>
+      <c r="D50" s="135">
+        <v>3959</v>
+      </c>
+      <c r="E50" s="135">
+        <v>71263714</v>
+      </c>
+      <c r="F50" s="135">
+        <v>69773086</v>
+      </c>
+      <c r="G50" s="135">
+        <v>1490628</v>
+      </c>
+      <c r="I50" s="3">
+        <f>E50/B50</f>
+        <v>372.98347150692962</v>
+      </c>
+      <c r="J50" s="26">
+        <f>I50*B33</f>
+        <v>12006217101.163296</v>
+      </c>
+      <c r="K50" s="26">
+        <f>J50*[2]About!$B$64</f>
+        <v>7460315126.3669386</v>
+      </c>
+      <c r="M50" s="3">
+        <f t="shared" si="0"/>
+        <v>168.47588242683079</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13">
+      <c r="A51" s="132">
+        <v>2024</v>
+      </c>
+      <c r="B51" s="135">
+        <v>186784</v>
+      </c>
+      <c r="C51" s="135">
+        <v>185153</v>
+      </c>
+      <c r="D51" s="135">
+        <v>1631</v>
+      </c>
+      <c r="E51" s="135">
+        <v>68848005</v>
+      </c>
+      <c r="F51" s="135">
+        <v>68225653</v>
+      </c>
+      <c r="G51" s="135">
+        <v>622352</v>
+      </c>
+      <c r="I51" s="3">
+        <f>E51/B51</f>
+        <v>368.59690872879906</v>
+      </c>
+      <c r="J51" s="26">
+        <f>I51*B34</f>
+        <v>11475066813.317791</v>
+      </c>
+      <c r="K51" s="26">
+        <f>J51*[2]About!$B$64</f>
+        <v>7130273740.8580894</v>
+      </c>
+      <c r="M51" s="3">
+        <f t="shared" si="0"/>
+        <v>166.67246659242764</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13">
+      <c r="A53" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="54" spans="1:13" ht="30">
+      <c r="A54" s="134" t="s">
+        <v>500</v>
+      </c>
+      <c r="B54" s="133" t="s">
+        <v>499</v>
+      </c>
+      <c r="C54" s="133" t="s">
+        <v>498</v>
+      </c>
+      <c r="D54" s="133" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13">
+      <c r="A55" s="132">
+        <v>2019</v>
+      </c>
+      <c r="B55" s="131">
+        <v>32980968</v>
+      </c>
+      <c r="C55" s="131">
+        <v>90385640</v>
+      </c>
+      <c r="D55" s="131">
+        <v>123366608</v>
+      </c>
+      <c r="F55">
+        <f>B55/D55</f>
+        <v>0.26734112686311357</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13">
+      <c r="A56" s="132">
+        <v>2020</v>
+      </c>
+      <c r="B56" s="131">
+        <v>25164038</v>
+      </c>
+      <c r="C56" s="131">
+        <v>42911044</v>
+      </c>
+      <c r="D56" s="131">
+        <v>68075082</v>
+      </c>
+      <c r="F56">
+        <f>B56/D56</f>
+        <v>0.36965123303119929</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13">
+      <c r="A57" s="132">
+        <v>2021</v>
+      </c>
+      <c r="B57" s="131">
+        <v>33146646</v>
+      </c>
+      <c r="C57" s="131">
+        <v>32043421</v>
+      </c>
+      <c r="D57" s="131">
+        <v>65190067</v>
+      </c>
+      <c r="F57">
+        <f>B57/D57</f>
+        <v>0.50846160351392189</v>
+      </c>
+    </row>
+    <row r="58" spans="1:13">
+      <c r="A58" s="132">
+        <v>2022</v>
+      </c>
+      <c r="B58" s="131">
+        <v>36328296</v>
+      </c>
+      <c r="C58" s="131">
+        <v>39609650</v>
+      </c>
+      <c r="D58" s="131">
+        <v>75937946</v>
+      </c>
+      <c r="F58">
+        <f>B58/D58</f>
+        <v>0.47839450384923499</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13">
+      <c r="A59" s="132">
+        <v>2023</v>
+      </c>
+      <c r="B59" s="131">
+        <v>32189676</v>
+      </c>
+      <c r="C59" s="131">
+        <v>68319015</v>
+      </c>
+      <c r="D59" s="131">
+        <v>100508691</v>
+      </c>
+      <c r="F59">
+        <f>B59/D59</f>
+        <v>0.32026758760593149</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13">
+      <c r="A60" s="132">
+        <v>2024</v>
+      </c>
+      <c r="B60" s="131">
+        <v>31131750</v>
+      </c>
+      <c r="C60" s="131">
+        <v>88926621</v>
+      </c>
+      <c r="D60" s="131">
+        <v>120058371</v>
+      </c>
+      <c r="F60">
+        <f>B60/D60</f>
+        <v>0.25930511750821605</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9438158E-C803-4774-ADE5-31C8503BC4B7}">
   <dimension ref="A1:Q31"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -5990,7 +7065,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8AABE4-9A7A-4FF9-8C38-25844DE09CA8}">
   <dimension ref="A1:AK15"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -7562,7 +8637,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EE2F069-6EF7-4399-A268-65FC5EA4C37A}">
   <sheetPr>
     <tabColor theme="3"/>
@@ -7710,8 +8785,8 @@
         <v>4</v>
       </c>
       <c r="B4" s="5">
-        <f>BAADTbVT_air!K17</f>
-        <v>147.99206308168749</v>
+        <f>'Air-Calcs'!M47</f>
+        <v>145.95406739643701</v>
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
@@ -7886,7 +8961,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05E0EE5E-AFD1-49CB-B732-B47A0DBCC6BF}">
   <sheetPr>
     <tabColor theme="3"/>
@@ -7962,7 +9037,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="41">
-        <f>BAADTbVT_air!L7</f>
+        <f>BAADTbVT_air!L9</f>
         <v>63.556825639903742</v>
       </c>
       <c r="C4" s="3"/>
@@ -8101,7 +9176,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
@@ -8529,7 +9604,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="5">
-        <f>BAADTbVT_air!K16</f>
+        <f>BAADTbVT_air!K18</f>
         <v>155.72981935122084</v>
       </c>
       <c r="C4" s="4">
@@ -8552,125 +9627,122 @@
         <f t="shared" si="0"/>
         <v>155.72981935122084</v>
       </c>
-      <c r="H4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
-      </c>
-      <c r="I4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
-      </c>
-      <c r="J4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
-      </c>
-      <c r="K4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+      <c r="H4" s="138" cm="1">
+        <f t="array" ref="H4:K4">TRANSPOSE('Air-Calcs'!M48:M51)</f>
+        <v>155.84487281959659</v>
+      </c>
+      <c r="I4" s="138">
+        <v>167.84077248261684</v>
+      </c>
+      <c r="J4" s="138">
+        <v>168.47588242683079</v>
+      </c>
+      <c r="K4" s="138">
+        <v>166.67246659242764</v>
       </c>
       <c r="L4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f>K4</f>
+        <v>166.67246659242764</v>
       </c>
       <c r="M4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" ref="M4:AK4" si="2">L4</f>
+        <v>166.67246659242764</v>
       </c>
       <c r="N4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" si="2"/>
+        <v>166.67246659242764</v>
       </c>
       <c r="O4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" si="2"/>
+        <v>166.67246659242764</v>
       </c>
       <c r="P4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" si="2"/>
+        <v>166.67246659242764</v>
       </c>
       <c r="Q4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" si="2"/>
+        <v>166.67246659242764</v>
       </c>
       <c r="R4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" si="2"/>
+        <v>166.67246659242764</v>
       </c>
       <c r="S4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" si="2"/>
+        <v>166.67246659242764</v>
       </c>
       <c r="T4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" si="2"/>
+        <v>166.67246659242764</v>
       </c>
       <c r="U4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" si="2"/>
+        <v>166.67246659242764</v>
       </c>
       <c r="V4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" si="2"/>
+        <v>166.67246659242764</v>
       </c>
       <c r="W4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" si="2"/>
+        <v>166.67246659242764</v>
       </c>
       <c r="X4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" si="2"/>
+        <v>166.67246659242764</v>
       </c>
       <c r="Y4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" si="2"/>
+        <v>166.67246659242764</v>
       </c>
       <c r="Z4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" si="2"/>
+        <v>166.67246659242764</v>
       </c>
       <c r="AA4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" si="2"/>
+        <v>166.67246659242764</v>
       </c>
       <c r="AB4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" si="2"/>
+        <v>166.67246659242764</v>
       </c>
       <c r="AC4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" si="2"/>
+        <v>166.67246659242764</v>
       </c>
       <c r="AD4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" si="2"/>
+        <v>166.67246659242764</v>
       </c>
       <c r="AE4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" si="2"/>
+        <v>166.67246659242764</v>
       </c>
       <c r="AF4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" si="2"/>
+        <v>166.67246659242764</v>
       </c>
       <c r="AG4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" si="2"/>
+        <v>166.67246659242764</v>
       </c>
       <c r="AH4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" si="2"/>
+        <v>166.67246659242764</v>
       </c>
       <c r="AI4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" si="2"/>
+        <v>166.67246659242764</v>
       </c>
       <c r="AJ4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" si="2"/>
+        <v>166.67246659242764</v>
       </c>
       <c r="AK4" s="4">
-        <f t="shared" si="0"/>
-        <v>155.72981935122084</v>
+        <f t="shared" si="2"/>
+        <v>166.67246659242764</v>
       </c>
     </row>
     <row r="5" spans="1:37">
@@ -8835,139 +9907,139 @@
         <v>337.61417769892506</v>
       </c>
       <c r="D6" s="4">
-        <f t="shared" ref="D6:AK6" si="2">C6</f>
+        <f t="shared" ref="D6:AK6" si="3">C6</f>
         <v>337.61417769892506</v>
       </c>
       <c r="E6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="F6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="G6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="H6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="I6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="J6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="K6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="L6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="M6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="N6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="O6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="P6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="Q6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="R6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="S6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="T6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="U6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="V6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="W6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="X6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="Y6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="Z6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="AA6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="AB6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="AC6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="AD6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="AE6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="AF6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="AG6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="AH6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="AI6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="AJ6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
       <c r="AK6" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>337.61417769892506</v>
       </c>
     </row>
@@ -9125,7 +10197,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
@@ -9541,7 +10613,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="41">
-        <f>BAADTbVT_air!L7</f>
+        <f>BAADTbVT_air!L9</f>
         <v>63.556825639903742</v>
       </c>
       <c r="C4" s="3">
@@ -19319,18 +20391,18 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{152A55CB-ED11-48EF-AA99-B206FDDEB829}">
-  <dimension ref="A1:P51"/>
+  <dimension ref="A1:P55"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9" style="8"/>
+    <col min="1" max="1" width="10" style="8" customWidth="1"/>
     <col min="2" max="2" width="13.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.7109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9" style="8"/>
-    <col min="9" max="9" width="11" style="8" customWidth="1"/>
+    <col min="3" max="3" width="23.28515625" style="8" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" style="8" customWidth="1"/>
+    <col min="5" max="5" width="23.140625" style="8" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" style="8" customWidth="1"/>
+    <col min="7" max="7" width="14.28515625" style="8" customWidth="1"/>
+    <col min="8" max="8" width="14.7109375" style="8" customWidth="1"/>
+    <col min="9" max="9" width="15.140625" style="8" customWidth="1"/>
     <col min="10" max="10" width="12.28515625" style="8" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="15.85546875" style="8" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="9.140625" style="8" bestFit="1" customWidth="1"/>
@@ -19341,1503 +20413,1645 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="str">
+        <f>_xlfn.TRANSLATE(A3)</f>
+        <v>Ministry of Land, Infrastructure, Transport and Tourism_Domestic International Air Transportation Performance by Year</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16">
+      <c r="A2" s="8" t="str">
+        <f t="shared" ref="A2:G2" si="0">_xlfn.TRANSLATE(A4)</f>
+        <v>Classification</v>
+      </c>
+      <c r="B2" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Passengers</v>
+      </c>
+      <c r="C2" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Passenger kilo (km)</v>
+      </c>
+      <c r="D2" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Cargo (tons)</v>
+      </c>
+      <c r="E2" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Cargo tonkilometer (km)</v>
+      </c>
+      <c r="F2" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Flights</v>
+      </c>
+      <c r="G2" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Kilometers (km)</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16">
+      <c r="A3" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:16">
-      <c r="A2" s="9" t="s">
+    <row r="4" spans="1:16">
+      <c r="A4" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B4" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C4" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D4" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E4" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F4" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G4" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="I2" s="10" t="s">
+      <c r="I4" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="11"/>
-    </row>
-    <row r="3" spans="1:16">
-      <c r="A3" s="12">
+      <c r="J4" s="11"/>
+    </row>
+    <row r="5" spans="1:16">
+      <c r="A5" s="12">
         <v>1989</v>
       </c>
-      <c r="B3" s="13">
+      <c r="B5" s="13">
         <v>17234880</v>
       </c>
-      <c r="C3" s="13">
+      <c r="C5" s="13">
         <v>32973999372</v>
       </c>
-      <c r="D3" s="13">
+      <c r="D5" s="13">
         <v>865713</v>
       </c>
-      <c r="E3" s="13">
+      <c r="E5" s="13">
         <v>4331431570</v>
       </c>
-      <c r="F3" s="13">
+      <c r="F5" s="13">
         <v>122857</v>
       </c>
-      <c r="G3" s="13">
+      <c r="G5" s="13">
         <v>240728926</v>
       </c>
-      <c r="I3" s="120" t="s">
+      <c r="I5" s="120" t="s">
         <v>20</v>
       </c>
-      <c r="J3" s="14" t="s">
+      <c r="J5" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="K3" s="14" t="s">
+      <c r="K5" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="L3" s="14" t="s">
+      <c r="L5" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="M3" s="14" t="s">
+      <c r="M5" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="N3" s="14" t="s">
+      <c r="N5" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="O3" s="14" t="s">
+      <c r="O5" s="14" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:16">
-      <c r="A4" s="12">
+    <row r="6" spans="1:16">
+      <c r="A6" s="12">
         <v>1990</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B6" s="13">
         <v>20690235</v>
       </c>
-      <c r="C4" s="13">
+      <c r="C6" s="13">
         <v>40415780780</v>
       </c>
-      <c r="D4" s="13">
+      <c r="D6" s="13">
         <v>959590</v>
       </c>
-      <c r="E4" s="13">
+      <c r="E6" s="13">
         <v>4626454321</v>
       </c>
-      <c r="F4" s="13">
+      <c r="F6" s="13">
         <v>139529</v>
       </c>
-      <c r="G4" s="13">
+      <c r="G6" s="13">
         <v>280656064</v>
       </c>
-      <c r="I4" s="121"/>
-      <c r="J4" s="15" t="e">
+      <c r="I6" s="121"/>
+      <c r="J6" s="15" t="e">
         <f>INDEX(B:B,MATCH(About!$B$42,$A:$A,0))</f>
         <v>#N/A</v>
       </c>
-      <c r="K4" s="15" t="e">
-        <f>INDEX(C:C,MATCH(About!$B$42,$A:$A,0))*N49</f>
+      <c r="K6" s="15" t="e">
+        <f>INDEX(C:C,MATCH(About!$B$42,$A:$A,0))*N53</f>
         <v>#N/A</v>
       </c>
-      <c r="L4" s="15">
-        <f>K16</f>
+      <c r="L6" s="15">
+        <f>K18</f>
         <v>155.72981935122084</v>
       </c>
-      <c r="M4" s="15">
+      <c r="M6" s="15">
         <v>259915924</v>
       </c>
-      <c r="N4" s="15">
+      <c r="N6" s="15">
         <v>161504217</v>
       </c>
-      <c r="O4" s="15">
-        <f>N4/L4</f>
+      <c r="O6" s="15">
+        <f>N6/L6</f>
         <v>1037079.5886930045</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16">
-      <c r="A5" s="12">
-        <v>1991</v>
-      </c>
-      <c r="B5" s="13">
-        <v>22523737</v>
-      </c>
-      <c r="C5" s="13">
-        <v>42968310434</v>
-      </c>
-      <c r="D5" s="13">
-        <v>986884</v>
-      </c>
-      <c r="E5" s="13">
-        <v>4548580506</v>
-      </c>
-      <c r="F5" s="13">
-        <v>150595</v>
-      </c>
-      <c r="G5" s="13">
-        <v>300479394</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16">
-      <c r="A6" s="12">
-        <v>1992</v>
-      </c>
-      <c r="B6" s="13">
-        <v>25811748</v>
-      </c>
-      <c r="C6" s="13">
-        <v>50453658708</v>
-      </c>
-      <c r="D6" s="13">
-        <v>1078832</v>
-      </c>
-      <c r="E6" s="13">
-        <v>5062484859</v>
-      </c>
-      <c r="F6" s="13">
-        <v>177627</v>
-      </c>
-      <c r="G6" s="13">
-        <v>347095622</v>
-      </c>
-      <c r="I6" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="J6" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="K6" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="L6" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="M6" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="N6" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="O6" s="14" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:16">
       <c r="A7" s="12">
-        <v>1993</v>
+        <v>1991</v>
       </c>
       <c r="B7" s="13">
-        <v>27201333</v>
+        <v>22523737</v>
       </c>
       <c r="C7" s="13">
-        <v>53138303731</v>
+        <v>42968310434</v>
       </c>
       <c r="D7" s="13">
-        <v>1223888</v>
+        <v>986884</v>
       </c>
       <c r="E7" s="13">
-        <v>6287703403</v>
+        <v>4548580506</v>
       </c>
       <c r="F7" s="13">
-        <v>201182</v>
+        <v>150595</v>
       </c>
       <c r="G7" s="13">
-        <v>371002537</v>
-      </c>
-      <c r="I7" s="121"/>
-      <c r="J7" s="15" t="e">
-        <f>INDEX(D:D,MATCH(About!$B$42,$A:$A,0))*O49</f>
-        <v>#N/A</v>
-      </c>
-      <c r="K7" s="15" t="e">
-        <f>INDEX(E:E,MATCH(About!$B$42,$A:$A,0))*O49</f>
-        <v>#N/A</v>
-      </c>
-      <c r="L7" s="15">
-        <f>O12</f>
-        <v>63.556825639903742</v>
-      </c>
-      <c r="M7" s="15">
-        <v>343226964</v>
-      </c>
-      <c r="N7" s="15">
-        <v>213271282</v>
-      </c>
-      <c r="O7" s="15">
-        <f>N7/L7</f>
-        <v>3355599.9666871186</v>
+        <v>300479394</v>
       </c>
     </row>
     <row r="8" spans="1:16">
       <c r="A8" s="12">
-        <v>1994</v>
+        <v>1992</v>
       </c>
       <c r="B8" s="13">
-        <v>31481845</v>
+        <v>25811748</v>
       </c>
       <c r="C8" s="13">
-        <v>60636514958</v>
+        <v>50453658708</v>
       </c>
       <c r="D8" s="13">
-        <v>1418923</v>
+        <v>1078832</v>
       </c>
       <c r="E8" s="13">
-        <v>7107986755</v>
+        <v>5062484859</v>
       </c>
       <c r="F8" s="13">
-        <v>214424</v>
+        <v>177627</v>
       </c>
       <c r="G8" s="13">
-        <v>416475276</v>
-      </c>
-      <c r="I8" s="8" t="s">
-        <v>33</v>
+        <v>347095622</v>
+      </c>
+      <c r="I8" s="120" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="K8" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="L8" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="M8" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="N8" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="O8" s="14" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:16">
       <c r="A9" s="12">
-        <v>1995</v>
+        <v>1993</v>
       </c>
       <c r="B9" s="13">
-        <v>35611282</v>
+        <v>27201333</v>
       </c>
       <c r="C9" s="13">
-        <v>69018847961</v>
+        <v>53138303731</v>
       </c>
       <c r="D9" s="13">
-        <v>1613469</v>
+        <v>1223888</v>
       </c>
       <c r="E9" s="13">
-        <v>8218439669</v>
+        <v>6287703403</v>
       </c>
       <c r="F9" s="13">
-        <v>234027</v>
+        <v>201182</v>
       </c>
       <c r="G9" s="13">
-        <v>468101617</v>
+        <v>371002537</v>
+      </c>
+      <c r="I9" s="121"/>
+      <c r="J9" s="15" t="e">
+        <f>INDEX(D:D,MATCH(About!$B$42,$A:$A,0))*O53</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K9" s="15" t="e">
+        <f>INDEX(E:E,MATCH(About!$B$42,$A:$A,0))*O53</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L9" s="15">
+        <f>O14</f>
+        <v>63.556825639903742</v>
+      </c>
+      <c r="M9" s="15">
+        <v>343226964</v>
+      </c>
+      <c r="N9" s="15">
+        <v>213271282</v>
+      </c>
+      <c r="O9" s="15">
+        <f>N9/L9</f>
+        <v>3355599.9666871186</v>
       </c>
     </row>
     <row r="10" spans="1:16">
       <c r="A10" s="12">
-        <v>1996</v>
+        <v>1994</v>
       </c>
       <c r="B10" s="13">
-        <v>39559043</v>
+        <v>31481845</v>
       </c>
       <c r="C10" s="13">
-        <v>78775501273</v>
+        <v>60636514958</v>
       </c>
       <c r="D10" s="13">
-        <v>1782337</v>
+        <v>1418923</v>
       </c>
       <c r="E10" s="13">
-        <v>9176947009</v>
+        <v>7107986755</v>
       </c>
       <c r="F10" s="13">
-        <v>254565</v>
+        <v>214424</v>
       </c>
       <c r="G10" s="13">
-        <v>528539658</v>
-      </c>
-      <c r="I10" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="K10" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="L10" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="M10" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="N10" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="O10" s="7" t="s">
-        <v>39</v>
+        <v>416475276</v>
+      </c>
+      <c r="I10" s="8" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:16">
       <c r="A11" s="12">
-        <v>1997</v>
+        <v>1995</v>
       </c>
       <c r="B11" s="13">
-        <v>42176926</v>
+        <v>35611282</v>
       </c>
       <c r="C11" s="13">
-        <v>83426879836</v>
+        <v>69018847961</v>
       </c>
       <c r="D11" s="13">
-        <v>2018393</v>
+        <v>1613469</v>
       </c>
       <c r="E11" s="13">
-        <v>10700851468</v>
+        <v>8218439669</v>
       </c>
       <c r="F11" s="13">
-        <v>277048</v>
+        <v>234027</v>
       </c>
       <c r="G11" s="13">
-        <v>591150615</v>
-      </c>
-      <c r="I11" s="122">
-        <v>2019</v>
-      </c>
-      <c r="J11" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="K11" s="16">
-        <v>523827</v>
-      </c>
-      <c r="L11" s="16">
-        <v>1723221</v>
-      </c>
-      <c r="M11" s="8">
-        <f>K11/SUM($K$11:$K$12)</f>
-        <v>0.96627258993084442</v>
-      </c>
-      <c r="N11" s="8">
-        <f>L11/SUM($L$11:$L$12)</f>
-        <v>0.5972427766459848</v>
-      </c>
-      <c r="O11" s="8">
-        <f>L11/K11</f>
-        <v>3.2896757899077369</v>
-      </c>
-      <c r="P11" s="8" t="s">
-        <v>41</v>
+        <v>468101617</v>
       </c>
     </row>
     <row r="12" spans="1:16">
       <c r="A12" s="12">
-        <v>1998</v>
+        <v>1996</v>
       </c>
       <c r="B12" s="13">
-        <v>33608780</v>
+        <v>39559043</v>
       </c>
       <c r="C12" s="13">
-        <v>62612530888</v>
+        <v>78775501273</v>
       </c>
       <c r="D12" s="13">
-        <v>1834298</v>
+        <v>1782337</v>
       </c>
       <c r="E12" s="13">
-        <v>9400102457</v>
+        <v>9176947009</v>
       </c>
       <c r="F12" s="13">
-        <v>248188</v>
+        <v>254565</v>
       </c>
       <c r="G12" s="13">
-        <v>489105234</v>
-      </c>
-      <c r="I12" s="122"/>
-      <c r="J12" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="K12" s="16">
-        <v>18284</v>
-      </c>
-      <c r="L12" s="16">
-        <v>1162073</v>
-      </c>
-      <c r="M12" s="8">
-        <f>K12/SUM($K$11:$K$12)</f>
-        <v>3.3727410069155576E-2</v>
-      </c>
-      <c r="N12" s="8">
-        <f>L12/SUM($L$11:$L$12)</f>
-        <v>0.4027572233540152</v>
-      </c>
-      <c r="O12" s="48">
-        <f>L12/K12</f>
-        <v>63.556825639903742</v>
+        <v>528539658</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="K12" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="L12" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="M12" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="N12" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="O12" s="7" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:16">
       <c r="A13" s="12">
-        <v>1999</v>
+        <v>1997</v>
       </c>
       <c r="B13" s="13">
-        <v>37894642</v>
+        <v>42176926</v>
       </c>
       <c r="C13" s="13">
-        <v>72436042000</v>
+        <v>83426879836</v>
       </c>
       <c r="D13" s="13">
-        <v>2112703</v>
+        <v>2018393</v>
       </c>
       <c r="E13" s="13">
-        <v>10898300517</v>
+        <v>10700851468</v>
       </c>
       <c r="F13" s="13">
-        <v>246910</v>
+        <v>277048</v>
       </c>
       <c r="G13" s="13">
-        <v>498569299</v>
+        <v>591150615</v>
+      </c>
+      <c r="I13" s="122">
+        <v>2019</v>
+      </c>
+      <c r="J13" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="K13" s="16">
+        <v>523827</v>
+      </c>
+      <c r="L13" s="16">
+        <v>1723221</v>
+      </c>
+      <c r="M13" s="8">
+        <f>K13/SUM($K$13:$K$14)</f>
+        <v>0.96627258993084442</v>
+      </c>
+      <c r="N13" s="8">
+        <f>L13/SUM($L$13:$L$14)</f>
+        <v>0.5972427766459848</v>
+      </c>
+      <c r="O13" s="8">
+        <f>L13/K13</f>
+        <v>3.2896757899077369</v>
+      </c>
+      <c r="P13" s="8" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:16">
       <c r="A14" s="12">
-        <v>2000</v>
+        <v>1998</v>
       </c>
       <c r="B14" s="13">
-        <v>41967169</v>
+        <v>33608780</v>
       </c>
       <c r="C14" s="13">
-        <v>83955503185</v>
+        <v>62612530888</v>
       </c>
       <c r="D14" s="13">
-        <v>2383581</v>
+        <v>1834298</v>
       </c>
       <c r="E14" s="13">
-        <v>12429945390</v>
+        <v>9400102457</v>
       </c>
       <c r="F14" s="13">
-        <v>273691</v>
+        <v>248188</v>
       </c>
       <c r="G14" s="13">
-        <v>561891020</v>
-      </c>
-      <c r="I14" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="K14" s="13"/>
+        <v>489105234</v>
+      </c>
+      <c r="I14" s="122"/>
+      <c r="J14" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="K14" s="16">
+        <v>18284</v>
+      </c>
+      <c r="L14" s="16">
+        <v>1162073</v>
+      </c>
+      <c r="M14" s="8">
+        <f>K14/SUM($K$13:$K$14)</f>
+        <v>3.3727410069155576E-2</v>
+      </c>
+      <c r="N14" s="8">
+        <f>L14/SUM($L$13:$L$14)</f>
+        <v>0.4027572233540152</v>
+      </c>
+      <c r="O14" s="48">
+        <f>L14/K14</f>
+        <v>63.556825639903742</v>
+      </c>
     </row>
     <row r="15" spans="1:16">
       <c r="A15" s="12">
-        <v>2001</v>
+        <v>1999</v>
       </c>
       <c r="B15" s="13">
-        <v>42161838</v>
+        <v>37894642</v>
       </c>
       <c r="C15" s="13">
-        <v>84544146258</v>
+        <v>72436042000</v>
       </c>
       <c r="D15" s="13">
-        <v>2294864</v>
+        <v>2112703</v>
       </c>
       <c r="E15" s="13">
-        <v>11326745204</v>
+        <v>10898300517</v>
       </c>
       <c r="F15" s="13">
-        <v>283914</v>
+        <v>246910</v>
       </c>
       <c r="G15" s="13">
-        <v>567756515</v>
-      </c>
-      <c r="I15" s="8" t="s">
-        <v>435</v>
+        <v>498569299</v>
       </c>
     </row>
     <row r="16" spans="1:16">
       <c r="A16" s="12">
-        <v>2002</v>
+        <v>2000</v>
       </c>
       <c r="B16" s="13">
-        <v>43965144</v>
+        <v>41967169</v>
       </c>
       <c r="C16" s="13">
-        <v>92174967638</v>
+        <v>83955503185</v>
       </c>
       <c r="D16" s="13">
-        <v>2509507</v>
+        <v>2383581</v>
       </c>
       <c r="E16" s="13">
-        <v>12606344764</v>
+        <v>12429945390</v>
       </c>
       <c r="F16" s="13">
-        <v>303032</v>
+        <v>273691</v>
       </c>
       <c r="G16" s="13">
-        <v>641000008</v>
-      </c>
-      <c r="I16" s="8">
-        <f>SUM(B49,I49)/SUM(C49,J49)*N49</f>
-        <v>155.72981935122084</v>
-      </c>
-      <c r="K16" s="48">
-        <f>I16</f>
-        <v>155.72981935122084</v>
-      </c>
+        <v>561891020</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="K16" s="13"/>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" s="12">
-        <v>2003</v>
+        <v>2001</v>
       </c>
       <c r="B17" s="13">
-        <v>42838812</v>
+        <v>42161838</v>
       </c>
       <c r="C17" s="13">
-        <v>82231019775</v>
+        <v>84544146258</v>
       </c>
       <c r="D17" s="13">
-        <v>2631359</v>
+        <v>2294864</v>
       </c>
       <c r="E17" s="13">
-        <v>11695819583</v>
+        <v>11326745204</v>
       </c>
       <c r="F17" s="13">
-        <v>310124</v>
+        <v>283914</v>
       </c>
       <c r="G17" s="13">
-        <v>615049182</v>
-      </c>
-      <c r="I17" s="8">
-        <f>SUM(B50,I50)/SUM(C50,J50)*N50</f>
-        <v>147.99206308168749</v>
-      </c>
-      <c r="K17" s="48">
-        <f>I17</f>
-        <v>147.99206308168749</v>
+        <v>567756515</v>
+      </c>
+      <c r="I17" s="8" t="s">
+        <v>435</v>
       </c>
     </row>
     <row r="18" spans="1:11">
       <c r="A18" s="12">
-        <v>2004</v>
+        <v>2002</v>
       </c>
       <c r="B18" s="13">
-        <v>45823588</v>
+        <v>43965144</v>
       </c>
       <c r="C18" s="13">
-        <v>96583257785</v>
+        <v>92174967638</v>
       </c>
       <c r="D18" s="13">
-        <v>2978118</v>
+        <v>2509507</v>
       </c>
       <c r="E18" s="13">
-        <v>13809815644</v>
+        <v>12606344764</v>
       </c>
       <c r="F18" s="13">
-        <v>313708</v>
+        <v>303032</v>
       </c>
       <c r="G18" s="13">
-        <v>688719258</v>
+        <v>641000008</v>
+      </c>
+      <c r="I18" s="8">
+        <f>SUM(B53,I53)/SUM(C53,J53)*N53</f>
+        <v>155.72981935122084</v>
+      </c>
+      <c r="K18" s="48">
+        <f>I18</f>
+        <v>155.72981935122084</v>
       </c>
     </row>
     <row r="19" spans="1:11">
       <c r="A19" s="12">
-        <v>2005</v>
+        <v>2003</v>
       </c>
       <c r="B19" s="13">
-        <v>46841441</v>
+        <v>42838812</v>
       </c>
       <c r="C19" s="13">
-        <v>101664000000</v>
+        <v>82231019775</v>
       </c>
       <c r="D19" s="13">
-        <v>2989203</v>
+        <v>2631359</v>
       </c>
       <c r="E19" s="13">
-        <v>13597859781</v>
+        <v>11695819583</v>
       </c>
       <c r="F19" s="13">
-        <v>314128</v>
+        <v>310124</v>
       </c>
       <c r="G19" s="13">
-        <v>697677439</v>
+        <v>615049182</v>
+      </c>
+      <c r="I19" s="8">
+        <f>SUM(B54,I54)/SUM(C54,J54)*N54</f>
+        <v>147.99206308168749</v>
+      </c>
+      <c r="K19" s="48">
+        <f>I19</f>
+        <v>147.99206308168749</v>
       </c>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="12">
-        <v>2006</v>
+        <v>2004</v>
       </c>
       <c r="B20" s="13">
-        <v>49888580</v>
+        <v>45823588</v>
       </c>
       <c r="C20" s="13">
-        <v>110791000000</v>
+        <v>96583257785</v>
       </c>
       <c r="D20" s="13">
-        <v>3208783</v>
+        <v>2978118</v>
       </c>
       <c r="E20" s="13">
-        <v>14730313293</v>
+        <v>13809815644</v>
       </c>
       <c r="F20" s="13">
-        <v>340637</v>
+        <v>313708</v>
       </c>
       <c r="G20" s="13">
-        <v>765599846</v>
+        <v>688719258</v>
       </c>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="12">
-        <v>2007</v>
+        <v>2005</v>
       </c>
       <c r="B21" s="13">
-        <v>53715079</v>
+        <v>46841441</v>
       </c>
       <c r="C21" s="13">
-        <v>121308000000</v>
+        <v>101664000000</v>
       </c>
       <c r="D21" s="13">
-        <v>3454508</v>
+        <v>2989203</v>
       </c>
       <c r="E21" s="13">
-        <v>15880213082</v>
+        <v>13597859781</v>
       </c>
       <c r="F21" s="13">
-        <v>386314</v>
+        <v>314128</v>
       </c>
       <c r="G21" s="13">
-        <v>860482950</v>
+        <v>697677439</v>
       </c>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="12">
-        <v>2008</v>
+        <v>2006</v>
       </c>
       <c r="B22" s="13">
-        <v>52331770</v>
+        <v>49888580</v>
       </c>
       <c r="C22" s="13">
-        <v>121563000000</v>
+        <v>110791000000</v>
       </c>
       <c r="D22" s="13">
-        <v>3251606</v>
+        <v>3208783</v>
       </c>
       <c r="E22" s="13">
-        <v>14948577845</v>
+        <v>14730313293</v>
       </c>
       <c r="F22" s="13">
-        <v>389484</v>
+        <v>340637</v>
       </c>
       <c r="G22" s="13">
-        <v>868323394</v>
+        <v>765599846</v>
       </c>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="12">
-        <v>2009</v>
+        <v>2007</v>
       </c>
       <c r="B23" s="13">
-        <v>51574629</v>
+        <v>53715079</v>
       </c>
       <c r="C23" s="13">
-        <v>116308000000</v>
+        <v>121308000000</v>
       </c>
       <c r="D23" s="13">
-        <v>3141146</v>
+        <v>3454508</v>
       </c>
       <c r="E23" s="13">
-        <v>14085183952</v>
+        <v>15880213082</v>
       </c>
       <c r="F23" s="13">
-        <v>379865</v>
+        <v>386314</v>
       </c>
       <c r="G23" s="13">
-        <v>790370533</v>
+        <v>860482950</v>
       </c>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="12">
-        <v>2010</v>
+        <v>2008</v>
       </c>
       <c r="B24" s="13">
-        <v>60277303</v>
+        <v>52331770</v>
       </c>
       <c r="C24" s="13">
-        <v>135771000000</v>
+        <v>121563000000</v>
       </c>
       <c r="D24" s="13">
-        <v>3588741</v>
+        <v>3251606</v>
       </c>
       <c r="E24" s="13">
-        <v>16376088401</v>
+        <v>14948577845</v>
       </c>
       <c r="F24" s="13">
-        <v>403296</v>
+        <v>389484</v>
       </c>
       <c r="G24" s="13">
-        <v>894995910</v>
+        <v>868323394</v>
       </c>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="12">
-        <v>2011</v>
+        <v>2009</v>
       </c>
       <c r="B25" s="13">
-        <v>63629352</v>
+        <v>51574629</v>
       </c>
       <c r="C25" s="13">
-        <v>148394000000</v>
+        <v>116308000000</v>
       </c>
       <c r="D25" s="13">
-        <v>3519237</v>
+        <v>3141146</v>
       </c>
       <c r="E25" s="13">
-        <v>16021369980</v>
+        <v>14085183952</v>
       </c>
       <c r="F25" s="13">
-        <v>432080</v>
+        <v>379865</v>
       </c>
       <c r="G25" s="13">
-        <v>984715383</v>
+        <v>790370533</v>
       </c>
     </row>
     <row r="26" spans="1:11">
       <c r="A26" s="12">
-        <v>2012</v>
+        <v>2010</v>
       </c>
       <c r="B26" s="13">
-        <v>69304162</v>
+        <v>60277303</v>
       </c>
       <c r="C26" s="13">
-        <v>162735000000</v>
+        <v>135771000000</v>
       </c>
       <c r="D26" s="13">
-        <v>3474057</v>
+        <v>3588741</v>
       </c>
       <c r="E26" s="13">
-        <v>15678617167</v>
+        <v>16376088401</v>
       </c>
       <c r="F26" s="13">
-        <v>469335</v>
+        <v>403296</v>
       </c>
       <c r="G26" s="13">
-        <v>1055832994</v>
+        <v>894995910</v>
       </c>
     </row>
     <row r="27" spans="1:11">
       <c r="A27" s="12">
-        <v>2013</v>
+        <v>2011</v>
       </c>
       <c r="B27" s="13">
-        <v>73340261</v>
+        <v>63629352</v>
       </c>
       <c r="C27" s="13">
-        <v>172963000000</v>
+        <v>148394000000</v>
       </c>
       <c r="D27" s="13">
-        <v>3498939</v>
+        <v>3519237</v>
       </c>
       <c r="E27" s="13">
-        <v>15657045872</v>
+        <v>16021369980</v>
       </c>
       <c r="F27" s="13">
-        <v>500738</v>
+        <v>432080</v>
       </c>
       <c r="G27" s="13">
-        <v>1116671455</v>
+        <v>984715383</v>
       </c>
     </row>
     <row r="28" spans="1:11">
       <c r="A28" s="12">
-        <v>2014</v>
+        <v>2012</v>
       </c>
       <c r="B28" s="13">
-        <v>81426297</v>
+        <v>69304162</v>
       </c>
       <c r="C28" s="13">
-        <v>183113000000</v>
+        <v>162735000000</v>
       </c>
       <c r="D28" s="13">
-        <v>3693861</v>
+        <v>3474057</v>
       </c>
       <c r="E28" s="13">
-        <v>16472894383</v>
+        <v>15678617167</v>
       </c>
       <c r="F28" s="13">
-        <v>536586</v>
+        <v>469335</v>
       </c>
       <c r="G28" s="13">
-        <v>1151922788</v>
+        <v>1055832994</v>
       </c>
     </row>
     <row r="29" spans="1:11">
       <c r="A29" s="12">
-        <v>2015</v>
+        <v>2013</v>
       </c>
       <c r="B29" s="13">
-        <v>89414538</v>
+        <v>73340261</v>
       </c>
       <c r="C29" s="13">
-        <v>198443000000</v>
+        <v>172963000000</v>
       </c>
       <c r="D29" s="13">
-        <v>3806553</v>
+        <v>3498939</v>
       </c>
       <c r="E29" s="13">
-        <v>16780475856</v>
+        <v>15657045872</v>
       </c>
       <c r="F29" s="13">
-        <v>570591</v>
+        <v>500738</v>
       </c>
       <c r="G29" s="13">
-        <v>1197486056</v>
+        <v>1116671455</v>
       </c>
     </row>
     <row r="30" spans="1:11">
       <c r="A30" s="12">
-        <v>2016</v>
+        <v>2014</v>
       </c>
       <c r="B30" s="13">
-        <v>103913732</v>
+        <v>81426297</v>
       </c>
       <c r="C30" s="13">
-        <v>224081000000</v>
+        <v>183113000000</v>
       </c>
       <c r="D30" s="13">
-        <v>4073795</v>
+        <v>3693861</v>
       </c>
       <c r="E30" s="13">
-        <v>17477169423</v>
+        <v>16472894383</v>
       </c>
       <c r="F30" s="13">
-        <v>629853</v>
+        <v>536586</v>
       </c>
       <c r="G30" s="13">
-        <v>1291889819</v>
+        <v>1151922788</v>
       </c>
     </row>
     <row r="31" spans="1:11">
       <c r="A31" s="12">
-        <v>2017</v>
+        <v>2015</v>
       </c>
       <c r="B31" s="13">
-        <v>109361974</v>
+        <v>89414538</v>
       </c>
       <c r="C31" s="13">
-        <v>243641000000</v>
+        <v>198443000000</v>
       </c>
       <c r="D31" s="13">
-        <v>4321641</v>
+        <v>3806553</v>
       </c>
       <c r="E31" s="13">
-        <v>18875336169</v>
+        <v>16780475856</v>
       </c>
       <c r="F31" s="13">
-        <v>653654</v>
+        <v>570591</v>
       </c>
       <c r="G31" s="13">
-        <v>1365679888</v>
+        <v>1197486056</v>
       </c>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="12">
-        <v>2018</v>
+        <v>2016</v>
       </c>
       <c r="B32" s="13">
-        <v>117525898</v>
+        <v>103913732</v>
       </c>
       <c r="C32" s="13">
-        <v>263629000000</v>
+        <v>224081000000</v>
       </c>
       <c r="D32" s="13">
-        <v>4441975</v>
+        <v>4073795</v>
       </c>
       <c r="E32" s="13">
-        <v>19447758637</v>
+        <v>17477169423</v>
       </c>
       <c r="F32" s="13">
-        <v>691521</v>
+        <v>629853</v>
       </c>
       <c r="G32" s="13">
-        <v>1455708646</v>
+        <v>1291889819</v>
       </c>
     </row>
     <row r="33" spans="1:16">
-      <c r="A33" s="17">
-        <v>2019</v>
-      </c>
-      <c r="B33" s="18">
-        <v>123366608</v>
-      </c>
-      <c r="C33" s="18">
-        <v>281755000000</v>
-      </c>
-      <c r="D33" s="18">
-        <v>4274717</v>
-      </c>
-      <c r="E33" s="18">
-        <v>18306326147</v>
-      </c>
-      <c r="F33" s="18">
-        <v>723592</v>
-      </c>
-      <c r="G33" s="18">
-        <v>1543833004</v>
+      <c r="A33" s="12">
+        <v>2017</v>
+      </c>
+      <c r="B33" s="13">
+        <v>109361974</v>
+      </c>
+      <c r="C33" s="13">
+        <v>243641000000</v>
+      </c>
+      <c r="D33" s="13">
+        <v>4321641</v>
+      </c>
+      <c r="E33" s="13">
+        <v>18875336169</v>
+      </c>
+      <c r="F33" s="13">
+        <v>653654</v>
+      </c>
+      <c r="G33" s="13">
+        <v>1365679888</v>
       </c>
     </row>
     <row r="34" spans="1:16">
       <c r="A34" s="12">
+        <v>2018</v>
+      </c>
+      <c r="B34" s="13">
+        <v>117525898</v>
+      </c>
+      <c r="C34" s="13">
+        <v>263629000000</v>
+      </c>
+      <c r="D34" s="13">
+        <v>4441975</v>
+      </c>
+      <c r="E34" s="13">
+        <v>19447758637</v>
+      </c>
+      <c r="F34" s="13">
+        <v>691521</v>
+      </c>
+      <c r="G34" s="13">
+        <v>1455708646</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16">
+      <c r="A35" s="17">
+        <v>2019</v>
+      </c>
+      <c r="B35" s="18">
+        <v>123366608</v>
+      </c>
+      <c r="C35" s="18">
+        <v>281755000000</v>
+      </c>
+      <c r="D35" s="18">
+        <v>4274717</v>
+      </c>
+      <c r="E35" s="18">
+        <v>18306326147</v>
+      </c>
+      <c r="F35" s="18">
+        <v>723592</v>
+      </c>
+      <c r="G35" s="18">
+        <v>1543833004</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16">
+      <c r="A36" s="12">
         <v>2020</v>
       </c>
-      <c r="B34" s="13">
+      <c r="B36" s="13">
         <v>39403960</v>
       </c>
-      <c r="C34" s="13">
+      <c r="C36" s="13">
         <v>62314352681</v>
       </c>
-      <c r="D34" s="13">
+      <c r="D36" s="13">
         <v>3252778</v>
       </c>
-      <c r="E34" s="13">
+      <c r="E36" s="13">
         <v>15811549626</v>
       </c>
-      <c r="F34" s="13">
+      <c r="F36" s="13">
         <v>339594</v>
       </c>
-      <c r="G34" s="13">
+      <c r="G36" s="13">
         <v>770665128</v>
-      </c>
-    </row>
-    <row r="35" spans="1:16">
-      <c r="A35" s="7" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="37" spans="1:16">
       <c r="A37" s="7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16">
+      <c r="A39" s="7" t="str">
+        <f>_xlfn.TRANSLATE(A41)</f>
+        <v>Aviation statistics Summary of passenger, supply, operation, and cargo data by airline</v>
+      </c>
+      <c r="B39" s="7"/>
+      <c r="C39" s="7"/>
+      <c r="D39" s="7"/>
+      <c r="E39" s="7"/>
+      <c r="F39" s="7"/>
+      <c r="G39" s="7" t="str">
+        <f t="shared" ref="G39:N39" si="1">_xlfn.TRANSLATE(G41)</f>
+        <v/>
+      </c>
+      <c r="H39" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="I39" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J39" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="K39" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="L39" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="M39" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="N39" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v>Ratio of national deaths to total</v>
+      </c>
+      <c r="O39" s="7"/>
+    </row>
+    <row r="40" spans="1:16">
+      <c r="A40" s="7" t="str">
+        <f t="shared" ref="A40:O40" si="2">_xlfn.TRANSLATE(A42)</f>
+        <v>Nationality History</v>
+      </c>
+      <c r="B40" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v>Supply (stone)</v>
+      </c>
+      <c r="C40" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v>Flights</v>
+      </c>
+      <c r="D40" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v>Passengers</v>
+      </c>
+      <c r="E40" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v>Cargo (tons)</v>
+      </c>
+      <c r="F40" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="G40" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H40" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v>Foreign Carriers</v>
+      </c>
+      <c r="I40" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v>Supply (stone)</v>
+      </c>
+      <c r="J40" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v>Flights</v>
+      </c>
+      <c r="K40" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v>Passengers</v>
+      </c>
+      <c r="L40" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v>Cargo (tons)</v>
+      </c>
+      <c r="M40" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="N40" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v>Passengers</v>
+      </c>
+      <c r="O40" s="7" t="str">
+        <f t="shared" si="2"/>
+        <v>Cargo (tons)</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16">
+      <c r="A41" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="N37" s="7" t="s">
+      <c r="N41" s="7" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="38" spans="1:16">
-      <c r="A38" s="9" t="s">
+    <row r="42" spans="1:16">
+      <c r="A42" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="B38" s="7" t="s">
+      <c r="B42" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C38" s="7" t="s">
+      <c r="C42" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D38" s="7" t="s">
+      <c r="D42" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="E38" s="7" t="s">
+      <c r="E42" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="H38" s="9" t="s">
+      <c r="H42" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="I38" s="7" t="s">
+      <c r="I42" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J38" s="7" t="s">
+      <c r="J42" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="K38" s="7" t="s">
+      <c r="K42" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="L38" s="7" t="s">
+      <c r="L42" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="N38" s="7" t="s">
+      <c r="N42" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="O38" s="7" t="s">
+      <c r="O42" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="P38" s="8">
-        <f>AVERAGE(O39:O49)</f>
+      <c r="P42" s="8">
+        <f>AVERAGE(O43:O53)</f>
         <v>0.72088835996183043</v>
-      </c>
-    </row>
-    <row r="39" spans="1:16">
-      <c r="A39" s="12">
-        <v>2009</v>
-      </c>
-      <c r="B39" s="16">
-        <v>58017647</v>
-      </c>
-      <c r="C39" s="16">
-        <v>292381</v>
-      </c>
-      <c r="D39" s="16">
-        <v>40387789</v>
-      </c>
-      <c r="E39" s="16">
-        <v>2378141</v>
-      </c>
-      <c r="H39" s="12">
-        <v>2009</v>
-      </c>
-      <c r="I39" s="16">
-        <v>16331104</v>
-      </c>
-      <c r="J39" s="16">
-        <v>87476</v>
-      </c>
-      <c r="K39" s="16">
-        <v>11579779</v>
-      </c>
-      <c r="L39" s="16">
-        <v>762743</v>
-      </c>
-      <c r="N39" s="8">
-        <f>D39/SUM(D39,K39)</f>
-        <v>0.77717296680114023</v>
-      </c>
-      <c r="O39" s="8">
-        <f>E39/SUM(E39,L39)</f>
-        <v>0.75715658394260976</v>
-      </c>
-    </row>
-    <row r="40" spans="1:16">
-      <c r="A40" s="12">
-        <v>2010</v>
-      </c>
-      <c r="B40" s="16">
-        <v>61312548</v>
-      </c>
-      <c r="C40" s="16">
-        <v>307880</v>
-      </c>
-      <c r="D40" s="16">
-        <v>47237514</v>
-      </c>
-      <c r="E40" s="16">
-        <v>2666460</v>
-      </c>
-      <c r="H40" s="12">
-        <v>2010</v>
-      </c>
-      <c r="I40" s="16">
-        <v>17358540</v>
-      </c>
-      <c r="J40" s="16">
-        <v>95417</v>
-      </c>
-      <c r="K40" s="16">
-        <v>13495430</v>
-      </c>
-      <c r="L40" s="16">
-        <v>922120</v>
-      </c>
-      <c r="N40" s="8">
-        <f t="shared" ref="N40:O50" si="0">D40/SUM(D40,K40)</f>
-        <v>0.7777906172307405</v>
-      </c>
-      <c r="O40" s="8">
-        <f t="shared" si="0"/>
-        <v>0.74304042267414971</v>
-      </c>
-    </row>
-    <row r="41" spans="1:16">
-      <c r="A41" s="12">
-        <v>2011</v>
-      </c>
-      <c r="B41" s="16">
-        <v>65976928</v>
-      </c>
-      <c r="C41" s="16">
-        <v>328216</v>
-      </c>
-      <c r="D41" s="16">
-        <v>49538896</v>
-      </c>
-      <c r="E41" s="16">
-        <v>2623974</v>
-      </c>
-      <c r="H41" s="12">
-        <v>2011</v>
-      </c>
-      <c r="I41" s="16">
-        <v>19538208</v>
-      </c>
-      <c r="J41" s="16">
-        <v>103853</v>
-      </c>
-      <c r="K41" s="16">
-        <v>14588820</v>
-      </c>
-      <c r="L41" s="16">
-        <v>895258</v>
-      </c>
-      <c r="N41" s="8">
-        <f t="shared" si="0"/>
-        <v>0.77250367064375103</v>
-      </c>
-      <c r="O41" s="8">
-        <f t="shared" si="0"/>
-        <v>0.74560983760093114</v>
-      </c>
-    </row>
-    <row r="42" spans="1:16">
-      <c r="A42" s="12">
-        <v>2012</v>
-      </c>
-      <c r="B42" s="16">
-        <v>70457208</v>
-      </c>
-      <c r="C42" s="16">
-        <v>355775</v>
-      </c>
-      <c r="D42" s="16">
-        <v>53874897</v>
-      </c>
-      <c r="E42" s="16">
-        <v>2556561</v>
-      </c>
-      <c r="H42" s="12">
-        <v>2012</v>
-      </c>
-      <c r="I42" s="16">
-        <v>21378152</v>
-      </c>
-      <c r="J42" s="16">
-        <v>113579</v>
-      </c>
-      <c r="K42" s="16">
-        <v>15982369</v>
-      </c>
-      <c r="L42" s="16">
-        <v>917497</v>
-      </c>
-      <c r="N42" s="8">
-        <f t="shared" si="0"/>
-        <v>0.77121393499711255</v>
-      </c>
-      <c r="O42" s="8">
-        <f t="shared" si="0"/>
-        <v>0.73590049446497441</v>
       </c>
     </row>
     <row r="43" spans="1:16">
       <c r="A43" s="12">
-        <v>2013</v>
+        <v>2009</v>
       </c>
       <c r="B43" s="16">
-        <v>73317719</v>
+        <v>58017647</v>
       </c>
       <c r="C43" s="16">
-        <v>375144</v>
+        <v>292381</v>
       </c>
       <c r="D43" s="16">
-        <v>56145585</v>
+        <v>40387789</v>
       </c>
       <c r="E43" s="16">
-        <v>2569156</v>
+        <v>2378141</v>
       </c>
       <c r="H43" s="12">
-        <v>2013</v>
+        <v>2009</v>
       </c>
       <c r="I43" s="16">
-        <v>23697631</v>
+        <v>16331104</v>
       </c>
       <c r="J43" s="16">
-        <v>125595</v>
+        <v>87476</v>
       </c>
       <c r="K43" s="16">
-        <v>17819459</v>
+        <v>11579779</v>
       </c>
       <c r="L43" s="16">
-        <v>929791</v>
+        <v>762743</v>
       </c>
       <c r="N43" s="8">
-        <f t="shared" si="0"/>
-        <v>0.7590826958745539</v>
+        <f>D43/SUM(D43,K43)</f>
+        <v>0.77717296680114023</v>
       </c>
       <c r="O43" s="8">
-        <f t="shared" si="0"/>
-        <v>0.73426548044311613</v>
+        <f>E43/SUM(E43,L43)</f>
+        <v>0.75715658394260976</v>
       </c>
     </row>
     <row r="44" spans="1:16">
       <c r="A44" s="12">
-        <v>2014</v>
+        <v>2010</v>
       </c>
       <c r="B44" s="16">
-        <v>77209328</v>
+        <v>61312548</v>
       </c>
       <c r="C44" s="16">
-        <v>391048</v>
+        <v>307880</v>
       </c>
       <c r="D44" s="16">
-        <v>60788552</v>
+        <v>47237514</v>
       </c>
       <c r="E44" s="16">
-        <v>2658483</v>
+        <v>2666460</v>
       </c>
       <c r="H44" s="12">
-        <v>2014</v>
+        <v>2010</v>
       </c>
       <c r="I44" s="16">
-        <v>27619692</v>
+        <v>17358540</v>
       </c>
       <c r="J44" s="16">
-        <v>145538</v>
+        <v>95417</v>
       </c>
       <c r="K44" s="16">
-        <v>21344930</v>
+        <v>13495430</v>
       </c>
       <c r="L44" s="16">
-        <v>1035379</v>
+        <v>922120</v>
       </c>
       <c r="N44" s="8">
-        <f t="shared" si="0"/>
-        <v>0.74011901747937581</v>
+        <f t="shared" ref="N44:O54" si="3">D44/SUM(D44,K44)</f>
+        <v>0.7777906172307405</v>
       </c>
       <c r="O44" s="8">
-        <f t="shared" si="0"/>
-        <v>0.71970284758878378</v>
+        <f t="shared" si="3"/>
+        <v>0.74304042267414971</v>
       </c>
     </row>
     <row r="45" spans="1:16">
       <c r="A45" s="12">
-        <v>2015</v>
+        <v>2011</v>
       </c>
       <c r="B45" s="16">
-        <v>84329502</v>
+        <v>65976928</v>
       </c>
       <c r="C45" s="16">
-        <v>420486</v>
+        <v>328216</v>
       </c>
       <c r="D45" s="16">
-        <v>68106765</v>
+        <v>49538896</v>
       </c>
       <c r="E45" s="16">
-        <v>2733091</v>
+        <v>2623974</v>
       </c>
       <c r="H45" s="12">
-        <v>2015</v>
+        <v>2011</v>
       </c>
       <c r="I45" s="16">
-        <v>28582396</v>
+        <v>19538208</v>
       </c>
       <c r="J45" s="16">
-        <v>150111</v>
+        <v>103853</v>
       </c>
       <c r="K45" s="16">
-        <v>22132049</v>
+        <v>14588820</v>
       </c>
       <c r="L45" s="16">
-        <v>1073461</v>
+        <v>895258</v>
       </c>
       <c r="N45" s="8">
-        <f t="shared" si="0"/>
-        <v>0.75473914140759868</v>
+        <f t="shared" si="3"/>
+        <v>0.77250367064375103</v>
       </c>
       <c r="O45" s="8">
-        <f t="shared" si="0"/>
-        <v>0.71799649656697184</v>
+        <f t="shared" si="3"/>
+        <v>0.74560983760093114</v>
       </c>
     </row>
     <row r="46" spans="1:16">
       <c r="A46" s="12">
-        <v>2016</v>
+        <v>2012</v>
       </c>
       <c r="B46" s="16">
-        <v>94085064</v>
+        <v>70457208</v>
       </c>
       <c r="C46" s="16">
-        <v>464495</v>
+        <v>355775</v>
       </c>
       <c r="D46" s="16">
-        <v>78956163</v>
+        <v>53874897</v>
       </c>
       <c r="E46" s="16">
-        <v>2886178</v>
+        <v>2556561</v>
       </c>
       <c r="H46" s="12">
-        <v>2016</v>
+        <v>2012</v>
       </c>
       <c r="I46" s="16">
-        <v>31928821</v>
+        <v>21378152</v>
       </c>
       <c r="J46" s="16">
-        <v>165364</v>
+        <v>113579</v>
       </c>
       <c r="K46" s="16">
-        <v>25933915</v>
+        <v>15982369</v>
       </c>
       <c r="L46" s="16">
-        <v>1187678</v>
+        <v>917497</v>
       </c>
       <c r="N46" s="8">
-        <f t="shared" si="0"/>
-        <v>0.75275149476006686</v>
+        <f t="shared" si="3"/>
+        <v>0.77121393499711255</v>
       </c>
       <c r="O46" s="8">
-        <f t="shared" si="0"/>
-        <v>0.70846343120620858</v>
+        <f t="shared" si="3"/>
+        <v>0.73590049446497441</v>
       </c>
     </row>
     <row r="47" spans="1:16">
       <c r="A47" s="12">
-        <v>2017</v>
+        <v>2013</v>
       </c>
       <c r="B47" s="16">
-        <v>101616268</v>
+        <v>73317719</v>
       </c>
       <c r="C47" s="16">
-        <v>497211</v>
+        <v>375144</v>
       </c>
       <c r="D47" s="16">
-        <v>85904545</v>
+        <v>56145585</v>
       </c>
       <c r="E47" s="16">
-        <v>3031848</v>
+        <v>2569156</v>
       </c>
       <c r="H47" s="12">
-        <v>2017</v>
+        <v>2013</v>
       </c>
       <c r="I47" s="16">
-        <v>30565057</v>
+        <v>23697631</v>
       </c>
       <c r="J47" s="16">
-        <v>156448</v>
+        <v>125595</v>
       </c>
       <c r="K47" s="16">
-        <v>24513986</v>
+        <v>17819459</v>
       </c>
       <c r="L47" s="16">
-        <v>1289793</v>
+        <v>929791</v>
       </c>
       <c r="N47" s="8">
-        <f t="shared" si="0"/>
-        <v>0.77799029041601719</v>
+        <f t="shared" si="3"/>
+        <v>0.7590826958745539</v>
       </c>
       <c r="O47" s="8">
-        <f t="shared" si="0"/>
-        <v>0.70155017503767669</v>
+        <f t="shared" si="3"/>
+        <v>0.73426548044311613</v>
       </c>
     </row>
     <row r="48" spans="1:16">
       <c r="A48" s="12">
-        <v>2018</v>
+        <v>2014</v>
       </c>
       <c r="B48" s="16">
-        <v>107630602</v>
+        <v>77209328</v>
       </c>
       <c r="C48" s="16">
-        <v>524690</v>
+        <v>391048</v>
       </c>
       <c r="D48" s="16">
-        <v>91273049</v>
+        <v>60788552</v>
       </c>
       <c r="E48" s="16">
-        <v>3069951</v>
+        <v>2658483</v>
       </c>
       <c r="H48" s="12">
-        <v>2018</v>
+        <v>2014</v>
       </c>
       <c r="I48" s="16">
-        <v>33353714</v>
+        <v>27619692</v>
       </c>
       <c r="J48" s="16">
-        <v>166833</v>
+        <v>145538</v>
       </c>
       <c r="K48" s="16">
-        <v>27217444</v>
+        <v>21344930</v>
       </c>
       <c r="L48" s="16">
-        <v>1372050</v>
+        <v>1035379</v>
       </c>
       <c r="N48" s="8">
-        <f t="shared" si="0"/>
-        <v>0.7702984998129766</v>
+        <f t="shared" si="3"/>
+        <v>0.74011901747937581</v>
       </c>
       <c r="O48" s="8">
-        <f t="shared" si="0"/>
-        <v>0.69111893491244147</v>
+        <f t="shared" si="3"/>
+        <v>0.71970284758878378</v>
       </c>
     </row>
     <row r="49" spans="1:16">
       <c r="A49" s="12">
-        <v>2019</v>
+        <v>2015</v>
       </c>
       <c r="B49" s="16">
-        <v>111528123</v>
+        <v>84329502</v>
       </c>
       <c r="C49" s="16">
-        <v>542111</v>
+        <v>420486</v>
       </c>
       <c r="D49" s="16">
-        <v>94245011</v>
+        <v>68106765</v>
       </c>
       <c r="E49" s="16">
-        <v>2885294</v>
+        <v>2733091</v>
       </c>
       <c r="H49" s="12">
-        <v>2019</v>
+        <v>2015</v>
       </c>
       <c r="I49" s="16">
-        <v>37076549</v>
+        <v>28582396</v>
       </c>
       <c r="J49" s="16">
-        <v>181481</v>
+        <v>150111</v>
       </c>
       <c r="K49" s="16">
-        <v>30041872</v>
+        <v>22132049</v>
       </c>
       <c r="L49" s="16">
-        <v>1389423</v>
-      </c>
-      <c r="N49" s="19">
-        <f t="shared" si="0"/>
-        <v>0.75828606145026578</v>
-      </c>
-      <c r="O49" s="19">
-        <f t="shared" si="0"/>
-        <v>0.67496725514227018</v>
-      </c>
-      <c r="P49" s="8" t="s">
-        <v>278</v>
+        <v>1073461</v>
+      </c>
+      <c r="N49" s="8">
+        <f t="shared" si="3"/>
+        <v>0.75473914140759868</v>
+      </c>
+      <c r="O49" s="8">
+        <f t="shared" si="3"/>
+        <v>0.71799649656697184</v>
       </c>
     </row>
     <row r="50" spans="1:16">
       <c r="A50" s="12">
+        <v>2016</v>
+      </c>
+      <c r="B50" s="16">
+        <v>94085064</v>
+      </c>
+      <c r="C50" s="16">
+        <v>464495</v>
+      </c>
+      <c r="D50" s="16">
+        <v>78956163</v>
+      </c>
+      <c r="E50" s="16">
+        <v>2886178</v>
+      </c>
+      <c r="H50" s="12">
+        <v>2016</v>
+      </c>
+      <c r="I50" s="16">
+        <v>31928821</v>
+      </c>
+      <c r="J50" s="16">
+        <v>165364</v>
+      </c>
+      <c r="K50" s="16">
+        <v>25933915</v>
+      </c>
+      <c r="L50" s="16">
+        <v>1187678</v>
+      </c>
+      <c r="N50" s="8">
+        <f t="shared" si="3"/>
+        <v>0.75275149476006686</v>
+      </c>
+      <c r="O50" s="8">
+        <f t="shared" si="3"/>
+        <v>0.70846343120620858</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16">
+      <c r="A51" s="12">
+        <v>2017</v>
+      </c>
+      <c r="B51" s="16">
+        <v>101616268</v>
+      </c>
+      <c r="C51" s="16">
+        <v>497211</v>
+      </c>
+      <c r="D51" s="16">
+        <v>85904545</v>
+      </c>
+      <c r="E51" s="16">
+        <v>3031848</v>
+      </c>
+      <c r="H51" s="12">
+        <v>2017</v>
+      </c>
+      <c r="I51" s="16">
+        <v>30565057</v>
+      </c>
+      <c r="J51" s="16">
+        <v>156448</v>
+      </c>
+      <c r="K51" s="16">
+        <v>24513986</v>
+      </c>
+      <c r="L51" s="16">
+        <v>1289793</v>
+      </c>
+      <c r="N51" s="8">
+        <f t="shared" si="3"/>
+        <v>0.77799029041601719</v>
+      </c>
+      <c r="O51" s="8">
+        <f t="shared" si="3"/>
+        <v>0.70155017503767669</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16">
+      <c r="A52" s="12">
+        <v>2018</v>
+      </c>
+      <c r="B52" s="16">
+        <v>107630602</v>
+      </c>
+      <c r="C52" s="16">
+        <v>524690</v>
+      </c>
+      <c r="D52" s="16">
+        <v>91273049</v>
+      </c>
+      <c r="E52" s="16">
+        <v>3069951</v>
+      </c>
+      <c r="H52" s="12">
+        <v>2018</v>
+      </c>
+      <c r="I52" s="16">
+        <v>33353714</v>
+      </c>
+      <c r="J52" s="16">
+        <v>166833</v>
+      </c>
+      <c r="K52" s="16">
+        <v>27217444</v>
+      </c>
+      <c r="L52" s="16">
+        <v>1372050</v>
+      </c>
+      <c r="N52" s="8">
+        <f t="shared" si="3"/>
+        <v>0.7702984998129766</v>
+      </c>
+      <c r="O52" s="8">
+        <f t="shared" si="3"/>
+        <v>0.69111893491244147</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16">
+      <c r="A53" s="12">
+        <v>2019</v>
+      </c>
+      <c r="B53" s="16">
+        <v>111528123</v>
+      </c>
+      <c r="C53" s="16">
+        <v>542111</v>
+      </c>
+      <c r="D53" s="16">
+        <v>94245011</v>
+      </c>
+      <c r="E53" s="16">
+        <v>2885294</v>
+      </c>
+      <c r="H53" s="12">
+        <v>2019</v>
+      </c>
+      <c r="I53" s="16">
+        <v>37076549</v>
+      </c>
+      <c r="J53" s="16">
+        <v>181481</v>
+      </c>
+      <c r="K53" s="16">
+        <v>30041872</v>
+      </c>
+      <c r="L53" s="16">
+        <v>1389423</v>
+      </c>
+      <c r="N53" s="19">
+        <f t="shared" si="3"/>
+        <v>0.75828606145026578</v>
+      </c>
+      <c r="O53" s="19">
+        <f t="shared" si="3"/>
+        <v>0.67496725514227018</v>
+      </c>
+      <c r="P53" s="8" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16">
+      <c r="A54" s="12">
         <v>2020</v>
       </c>
-      <c r="B50" s="16">
+      <c r="B54" s="16">
         <v>48876694</v>
       </c>
-      <c r="C50" s="16">
+      <c r="C54" s="16">
         <v>275368</v>
       </c>
-      <c r="D50" s="16">
+      <c r="D54" s="16">
         <v>34952212</v>
       </c>
-      <c r="E50" s="16">
+      <c r="E54" s="16">
         <v>2346383</v>
       </c>
-      <c r="H50" s="12">
+      <c r="H54" s="12">
         <v>2020</v>
       </c>
-      <c r="I50" s="16">
+      <c r="I54" s="16">
         <v>8166640</v>
       </c>
-      <c r="J50" s="16">
+      <c r="J54" s="16">
         <v>64229</v>
       </c>
-      <c r="K50" s="16">
+      <c r="K54" s="16">
         <v>4719167</v>
       </c>
-      <c r="L50" s="16">
+      <c r="L54" s="16">
         <v>906395</v>
       </c>
-      <c r="N50" s="8">
-        <f t="shared" si="0"/>
+      <c r="N54" s="8">
+        <f t="shared" si="3"/>
         <v>0.88104353518943723</v>
       </c>
-      <c r="O50" s="8">
-        <f t="shared" si="0"/>
+      <c r="O54" s="8">
+        <f t="shared" si="3"/>
         <v>0.72134741442545414</v>
       </c>
     </row>
-    <row r="51" spans="1:16">
-      <c r="B51" s="16"/>
-      <c r="C51" s="16"/>
-      <c r="D51" s="16"/>
-      <c r="E51" s="16"/>
+    <row r="55" spans="1:16">
+      <c r="B55" s="16"/>
+      <c r="C55" s="16"/>
+      <c r="D55" s="16"/>
+      <c r="E55" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="I3:I4"/>
-    <mergeCell ref="I6:I7"/>
-    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="I8:I9"/>
+    <mergeCell ref="I13:I14"/>
   </mergeCells>
   <phoneticPr fontId="42" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -26304,6 +27518,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
     <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
@@ -26447,22 +27676,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{63D16A6B-8B1B-4121-BE38-0F3E968A7BF0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30D49544-8BCC-440A-9096-15397E5D5534}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1139C0F6-B00C-4379-81CA-44285F52FF2E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -26478,21 +27709,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30D49544-8BCC-440A-9096-15397E5D5534}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{63D16A6B-8B1B-4121-BE38-0F3E968A7BF0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>